<commit_message>
Keep plan notes beside products and explain that fungal and weed goals do not include chemicals.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/pd_master_application_guide.xlsx
+++ b/data/pd_master_application_guide.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'calendar_intervals'!$A$1:$Q$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'usage_guide_rates'!$A$1:$F$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'calculator_rates'!$A$1:$AX$153</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'program_notes'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'program_notes'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -382,8 +382,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProgramNotes" displayName="ProgramNotes" ref="A1:D13" headerRowCount="1">
-  <autoFilter ref="A1:D13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProgramNotes" displayName="ProgramNotes" ref="A1:D15" headerRowCount="1">
+  <autoFilter ref="A1:D15"/>
   <tableColumns count="4">
     <tableColumn id="1" name="note_id"/>
     <tableColumn id="2" name="applies_when"/>
@@ -34832,10 +34832,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
@@ -34906,209 +34906,245 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>humate_top_of_soil</t>
+          <t>fungal_no_chemical_fungicides</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Humate granules (513) on the plan</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>513</t>
-        </is>
-      </c>
+          <t>Fungal issues selected</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Spread Humate granules on the top layer of soil, under mulch, or dug in. They do not need to be watered in.</t>
+          <t>This plan does not include chemical fungicides. We support plant and soil health so lawns and gardens can resist disease, and we ease high-nitrogen feeds in summer.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>ffr_alternate_activ8</t>
+          <t>weed_suppression_no_chemicals</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Flowers, Fruits &amp; Roots liquid plus Activ8Mate or Activ8EXTRA</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>721, A8M, A8X</t>
-        </is>
-      </c>
+          <t>Weed suppression through dominance selected</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Alternate between Flowers, Fruits &amp; Roots and Activ8 each feed. FFR is for flowering/fruiting; Activ8 is the regular feed. Do not mix those two in the same sprayer.</t>
+          <t>This plan does not include chemical weed killers. We support thicker, healthier growth so lawns and gardens can crowd weeds out. Chemical products are on https://www.plantdoctor.com.au/weed-and-pest-control</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>mixable_same_day</t>
+          <t>humate_top_of_soil</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Two or more mix_together concentrates</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr"/>
+          <t>Humate granules (513) on the plan</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>513</t>
+        </is>
+      </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Mix mixable concentrates in one sprayer on the same day. Do not add iron to that tank. Jar test if it is a new combination.</t>
+          <t>Spread Humate granules on the top layer of soil, under mulch, or dug in. They do not need to be watered in.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>iron_separate_day</t>
+          <t>ffr_alternate_activ8</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Liquid iron plus seaweed, humic, wetter, or Activ8</t>
+          <t>Flowers, Fruits &amp; Roots liquid plus Activ8Mate or Activ8EXTRA</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>LIR, LEN, MG, 547, 846</t>
+          <t>721, A8M, A8X</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Liquid iron is on a different day from seaweed, humic, wetter, and Activ8. Do not mix them in the same sprayer.</t>
+          <t>Alternate between Flowers, Fruits &amp; Roots and Activ8 each feed. FFR is for flowering/fruiting; Activ8 is the regular feed. Do not mix those two in the same sprayer.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>lime_wait_before_iron</t>
+          <t>mixable_same_day</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Lime or dolomite and an iron product</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>LIMEGr, DOL</t>
-        </is>
-      </c>
+          <t>Two or more mix_together concentrates</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Wait 42 days after lime or dolomite before applying iron.</t>
+          <t>Mix mixable concentrates in one sprayer on the same day. Do not add iron to that tank. Jar test if it is a new combination.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>iron_gap_days</t>
+          <t>iron_separate_day</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Iron with seaweed / humic / wetter / Activ8</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr"/>
+          <t>Liquid iron plus seaweed, humic, wetter, or Activ8</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>LIR, LEN, MG, 547, 846</t>
+        </is>
+      </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Keep liquid iron at least 3 days away from seaweed, humic, wetter, and Activ8.</t>
+          <t>Liquid iron is on a different day from seaweed, humic, wetter, and Activ8. Do not mix them in the same sprayer.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>volcamin_no_badges</t>
+          <t>lime_wait_before_iron</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin (557)</t>
+          <t>Lime or dolomite and an iron product</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>LIMEGr, DOL</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin has no mix, apply-independently, or water-in badges. Incorporate into soil, potting mix, or the root zone.</t>
+          <t>Wait 42 days after lime or dolomite before applying iron.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>stimulizer_iron_exception</t>
+          <t>iron_gap_days</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Tank-mixing</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>STM</t>
-        </is>
-      </c>
+          <t>Iron with seaweed / humic / wetter / Activ8</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Stimulizer is the only product the usage guide says can be tank-mixed with iron.</t>
+          <t>Keep liquid iron at least 3 days away from seaweed, humic, wetter, and Activ8.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>default_home_rate</t>
+          <t>volcamin_no_badges</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>No product-specific rate</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr"/>
+          <t>VolcaMin (557)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>557</t>
+        </is>
+      </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Unless otherwise specified, apply 10 mL per 10 m² (100 mL per 100 m²) of lawn or garden.</t>
+          <t>VolcaMin has no mix, apply-independently, or water-in badges. Incorporate into soil, potting mix, or the root zone.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>stimulizer_iron_exception</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Tank-mixing</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>STM</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Stimulizer is the only product the usage guide says can be tank-mixed with iron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>default_home_rate</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>No product-specific rate</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Unless otherwise specified, apply 10 mL per 10 m² (100 mL per 100 m²) of lawn or garden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>source</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Always</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Joined from Product Usage Guide (Aug 2025), PD application rates sheet, schedule_intervals.csv, and the product catalog. Follow the label.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D13"/>
+  <autoFilter ref="A1:D15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Let customers pick South, North, or East coast so winter cadence matches where they are.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/pd_master_application_guide.xlsx
+++ b/data/pd_master_application_guide.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'calendar_intervals'!$A$1:$Q$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'usage_guide_rates'!$A$1:$F$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'calculator_rates'!$A$1:$AX$153</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'program_notes'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'program_notes'!$A$1:$D$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -382,8 +382,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProgramNotes" displayName="ProgramNotes" ref="A1:D15" headerRowCount="1">
-  <autoFilter ref="A1:D15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProgramNotes" displayName="ProgramNotes" ref="A1:D17" headerRowCount="1">
+  <autoFilter ref="A1:D17"/>
   <tableColumns count="4">
     <tableColumn id="1" name="note_id"/>
     <tableColumn id="2" name="applies_when"/>
@@ -34832,7 +34832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -34884,267 +34884,303 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>garden_natives_half_strength</t>
+          <t>winter_east_coast_june_july</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Garden selected</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>SWS, A8M</t>
-        </is>
-      </c>
+          <t>East coast selected, year-round sprays (cadence 42 days or less)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr"/>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>For natives and other sensitive plants, use Seaweed Secrets and Activ8Mate at half strength.</t>
+          <t>Keep applying through winter, just less often. On the east coast winter is shorter — usually June and July, when nights dip below 10°C.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>fungal_no_chemical_fungicides</t>
+          <t>winter_north_usual_cadence</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Fungal issues selected</t>
+          <t>North selected, year-round sprays (cadence 42 days or less)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>This plan does not include chemical fungicides. We support plant and soil health so lawns and gardens can resist disease, and we ease high-nitrogen feeds in summer.</t>
+          <t>Nights rarely drop below 10°C in the north, so this plan keeps the usual cadence year-round.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>weed_suppression_no_chemicals</t>
+          <t>garden_natives_half_strength</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Weed suppression through dominance selected</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr"/>
+          <t>Garden selected</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>SWS, A8M</t>
+        </is>
+      </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>This plan does not include chemical weed killers. We support thicker, healthier growth so lawns and gardens can crowd weeds out. Chemical products are on https://www.plantdoctor.com.au/weed-and-pest-control</t>
+          <t>For natives and other sensitive plants, use Seaweed Secrets and Activ8Mate at half strength.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>humate_top_of_soil</t>
+          <t>fungal_no_chemical_fungicides</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Humate granules (513) on the plan</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>513</t>
-        </is>
-      </c>
+          <t>Fungal issues selected</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Spread Humate granules on the top layer of soil, under mulch, or dug in. They do not need to be watered in.</t>
+          <t>This plan does not include chemical fungicides. We support plant and soil health so lawns and gardens can resist disease, and we ease high-nitrogen feeds in summer.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>ffr_alternate_activ8</t>
+          <t>weed_suppression_no_chemicals</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Flowers, Fruits &amp; Roots liquid plus Activ8Mate or Activ8EXTRA</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>721, A8M, A8X</t>
-        </is>
-      </c>
+          <t>Weed suppression through dominance selected</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Alternate between Flowers, Fruits &amp; Roots and Activ8 each feed. FFR is for flowering/fruiting; Activ8 is the regular feed. Do not mix those two in the same sprayer.</t>
+          <t>This plan does not include chemical weed killers. We support thicker, healthier growth so lawns and gardens can crowd weeds out. Chemical products are on https://www.plantdoctor.com.au/weed-and-pest-control</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>mixable_same_day</t>
+          <t>humate_top_of_soil</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Two or more mix_together concentrates</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr"/>
+          <t>Humate granules (513) on the plan</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>513</t>
+        </is>
+      </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Mix mixable concentrates in one sprayer on the same day. Do not add iron to that tank. Jar test if it is a new combination.</t>
+          <t>Spread Humate granules on the top layer of soil, under mulch, or dug in. They do not need to be watered in.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>iron_separate_day</t>
+          <t>ffr_alternate_activ8</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Liquid iron plus seaweed, humic, wetter, or Activ8</t>
+          <t>Flowers, Fruits &amp; Roots liquid plus Activ8Mate or Activ8EXTRA</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>LIR, LEN, MG, 547, 846</t>
+          <t>721, A8M, A8X</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Liquid iron is on a different day from seaweed, humic, wetter, and Activ8. Do not mix them in the same sprayer.</t>
+          <t>Alternate between Flowers, Fruits &amp; Roots and Activ8 each feed. FFR is for flowering/fruiting; Activ8 is the regular feed. Do not mix those two in the same sprayer.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>lime_wait_before_iron</t>
+          <t>mixable_same_day</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Lime or dolomite and an iron product</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>LIMEGr, DOL</t>
-        </is>
-      </c>
+          <t>Two or more mix_together concentrates</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Wait 42 days after lime or dolomite before applying iron.</t>
+          <t>Mix mixable concentrates in one sprayer on the same day. Do not add iron to that tank. Jar test if it is a new combination.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>iron_gap_days</t>
+          <t>iron_separate_day</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Iron with seaweed / humic / wetter / Activ8</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr"/>
+          <t>Liquid iron plus seaweed, humic, wetter, or Activ8</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>LIR, LEN, MG, 547, 846</t>
+        </is>
+      </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Keep liquid iron at least 3 days away from seaweed, humic, wetter, and Activ8.</t>
+          <t>Liquid iron is on a different day from seaweed, humic, wetter, and Activ8. Do not mix them in the same sprayer.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>volcamin_no_badges</t>
+          <t>lime_wait_before_iron</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin (557)</t>
+          <t>Lime or dolomite and an iron product</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>LIMEGr, DOL</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin has no mix, apply-independently, or water-in badges. Incorporate into soil, potting mix, or the root zone.</t>
+          <t>Wait 42 days after lime or dolomite before applying iron.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>stimulizer_iron_exception</t>
+          <t>iron_gap_days</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Tank-mixing</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>STM</t>
-        </is>
-      </c>
+          <t>Iron with seaweed / humic / wetter / Activ8</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Stimulizer is the only product the usage guide says can be tank-mixed with iron.</t>
+          <t>Keep liquid iron at least 3 days away from seaweed, humic, wetter, and Activ8.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>default_home_rate</t>
+          <t>volcamin_no_badges</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>No product-specific rate</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr"/>
+          <t>VolcaMin (557)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>557</t>
+        </is>
+      </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Unless otherwise specified, apply 10 mL per 10 m² (100 mL per 100 m²) of lawn or garden.</t>
+          <t>VolcaMin has no mix, apply-independently, or water-in badges. Incorporate into soil, potting mix, or the root zone.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>stimulizer_iron_exception</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Tank-mixing</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>STM</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Stimulizer is the only product the usage guide says can be tank-mixed with iron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>default_home_rate</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>No product-specific rate</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Unless otherwise specified, apply 10 mL per 10 m² (100 mL per 100 m²) of lawn or garden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>source</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Always</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Joined from Product Usage Guide (Aug 2025), PD application rates sheet, schedule_intervals.csv, and the product catalog. Follow the label.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D15"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -35281,7 +35317,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>growing_season skips typical temperate winter; year_round eases to about half cadence in June–August.</t>
+          <t>growing_season skips the region's winter; year_round eases to about half cadence in winter months (south Jun–Aug, east coast Jun–Jul, north no winter slowdown).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recommend fuller keep-it-healthy programs and fix broken product buy-now links.
Lawn plans that tick most goals now use the Pro Pack plus Champion and soil extras. Garden plans keep one Flowers Fruits & Roots form and add Roots, Shoots & Leaves granules when pushing for best results.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/pd_master_application_guide.xlsx
+++ b/data/pd_master_application_guide.xlsx
@@ -4788,7 +4788,7 @@
       <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>https://www.plantdoctor.com.au/iron-chelate-fertiliser</t>
+          <t>https://www.plantdoctor.com.au/kendon-iron-chelate</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
@@ -5659,7 +5659,7 @@
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>https://www.plantdoctor.com.au/micronised-gypsum-liquid-clay-buster</t>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
@@ -6240,7 +6240,7 @@
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>https://www.plantdoctor.com.au/neem-granules-fertiliser</t>
+          <t>https://www.plantdoctor.com.au/neem-fertiliser-slow-release-granules-1-2mm</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
@@ -7219,7 +7219,7 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>https://www.plantdoctor.com.au/activ8mate-liquid-fertiliser-inoculant-for-use-on</t>
+          <t>https://www.plantdoctor.com.au/activ8extra-high-nitrogen-liquid-lawn-fertiliser-p</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -12840,7 +12840,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>https://www.plantdoctor.com.au/activ8extra-boosted-liquid-fertiliser-and-inoculan</t>
+          <t>https://www.plantdoctor.com.au/activ8extra-high-nitrogen-liquid-lawn-fertiliser-p</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
@@ -12926,7 +12926,7 @@
       <c r="AT2" s="4" t="inlineStr"/>
       <c r="AU2" s="4" t="inlineStr">
         <is>
-          <t>https://www.plantdoctor.com.au/activ8extra-boosted-liquid-fertiliser-and-inoculan</t>
+          <t>https://www.plantdoctor.com.au/activ8extra-high-nitrogen-liquid-lawn-fertiliser-p</t>
         </is>
       </c>
       <c r="AV2" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Give liquid gypsum the product-page rates so the calendar shows a real amount.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/pd_master_application_guide.xlsx
+++ b/data/pd_master_application_guide.xlsx
@@ -18,8 +18,8 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'products'!$A$1:$AO$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'calendar_intervals'!$A$1:$Q$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'usage_guide_rates'!$A$1:$F$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'calculator_rates'!$A$1:$AX$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'usage_guide_rates'!$A$1:$F$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'calculator_rates'!$A$1:$AX$162</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'program_notes'!$A$1:$D$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -308,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="UsageGuideRates" displayName="UsageGuideRates" ref="A1:F80" headerRowCount="1">
-  <autoFilter ref="A1:F80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="UsageGuideRates" displayName="UsageGuideRates" ref="A1:F85" headerRowCount="1">
+  <autoFilter ref="A1:F85"/>
   <tableColumns count="6">
     <tableColumn id="1" name="sku"/>
     <tableColumn id="2" name="guide_name"/>
@@ -323,8 +323,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CalculatorRates" displayName="CalculatorRates" ref="A1:AX153" headerRowCount="1">
-  <autoFilter ref="A1:AX153"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CalculatorRates" displayName="CalculatorRates" ref="A1:AX162" headerRowCount="1">
+  <autoFilter ref="A1:AX162"/>
   <tableColumns count="50">
     <tableColumn id="1" name="sku"/>
     <tableColumn id="2" name="Product Name"/>
@@ -5700,7 +5700,7 @@
       </c>
       <c r="R26" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 2–4 weeks as required; higher rates on heavy clay. Do not tank-mix with iron. Not for drippers.</t>
+          <t>Home garden: 45 mL in 9 L water, apply 1 L/m² (500 mL per 100 m²) every 2–4 weeks. Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers.</t>
         </is>
       </c>
       <c r="S26" s="4" t="inlineStr">
@@ -5723,9 +5723,9 @@
           <t>1</t>
         </is>
       </c>
-      <c r="W26" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="W26" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="X26" s="10" t="inlineStr">
@@ -5755,19 +5755,39 @@
       </c>
       <c r="AC26" s="4" t="inlineStr">
         <is>
-          <t>Varies by application type.</t>
-        </is>
-      </c>
-      <c r="AD26" s="4" t="inlineStr"/>
+          <t>Home garden: 45 mL in 9 L water, apply 1 L/m² (500 mL per 100 m²). Soil ameliorant or fertigation: 10–50 L/ha. Foliar: 1 L per 100 L water, up to 5–7 L/ha depending on crop.</t>
+        </is>
+      </c>
+      <c r="AD26" s="4" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
       <c r="AE26" s="4" t="inlineStr">
         <is>
-          <t>Shake well before use and maintain constant agitation. Can be applied through fertigation, watering cans or spray equipment. A coarse filter is recommended, and a jar test should be performed before mixing. Not suitable for drippers.</t>
-        </is>
-      </c>
-      <c r="AF26" s="4" t="inlineStr"/>
-      <c r="AG26" s="4" t="inlineStr"/>
-      <c r="AH26" s="4" t="inlineStr"/>
-      <c r="AI26" s="4" t="inlineStr"/>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Will pass a 200-micron filter under ideal conditions; a coarse inline filter (500 micron / 35 mesh) is recommended. Drench with a watering can or equipment that can take larger particles. Not suitable for drippers. Foliar use can leave a visible residue on leaves and fruit. Jar test before mixing. Liquid inject minimum dilution 1-part product to 3-parts water. Store cool and keep sealed.</t>
+        </is>
+      </c>
+      <c r="AF26" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks</t>
+        </is>
+      </c>
+      <c r="AG26" s="4" t="inlineStr">
+        <is>
+          <t>Home garden: 45 mL in 9 L water; apply 1 L of mix per m² (500 mL product per 100 m²).</t>
+        </is>
+      </c>
+      <c r="AH26" s="4" t="inlineStr">
+        <is>
+          <t>500 mL / 100 m²</t>
+        </is>
+      </c>
+      <c r="AI26" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3. | Use higher rates for heavy clay (soil amelioration). Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
       <c r="AJ26" s="4" t="inlineStr">
         <is>
           <t>0</t>
@@ -5775,7 +5795,7 @@
       </c>
       <c r="AK26" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 2–4 weeks as required; higher rates on heavy clay. Do not tank-mix with iron. Not for drippers. | Shake well before use and maintain constant agitation. Can be applied through fertigation, watering cans or spray equipment. A coarse filter is recommended, and a jar test should be performed before mixing. Not suitable for drippers.</t>
+          <t>Home garden: 45 mL in 9 L water, apply 1 L/m² (500 mL per 100 m²) every 2–4 weeks. Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers. | Shake or stir well before use and keep agitating. Pre-mix slowly. Will pass a 200-micron filter under ideal conditions; a coarse inline filter (500 micron / 35 mesh) is recommended. Drench with a watering can or equipment that can take larger particles. Not suitable for drippers. Foliar use can leave a visible residue on leaves and fruit. Jar test before mixing. Liquid inject minimum dilution 1-part product to 3-parts water. Store cool and keep sealed. | Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3. | Use higher rates for heavy clay (soil amelioration). Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
         </is>
       </c>
       <c r="AL26" s="4" t="inlineStr">
@@ -5795,7 +5815,7 @@
       </c>
       <c r="AO26" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -9825,9 +9845,9 @@
           <t>1</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
+      <c r="L28" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
       <c r="M28" s="10" t="inlineStr">
@@ -9852,7 +9872,7 @@
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 2–4 weeks as required; higher rates on heavy clay. Do not tank-mix with iron. Not for drippers.</t>
+          <t>Home garden: 45 mL in 9 L water, apply 1 L/m² (500 mL per 100 m²) every 2–4 weeks. Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers.</t>
         </is>
       </c>
     </row>
@@ -10132,7 +10152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11651,7 +11671,7 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Apply at 1 L/m²</t>
+          <t>Apply 1 L/m² every 2–4 weeks (500 mL per 100 m²)</t>
         </is>
       </c>
     </row>
@@ -11681,7 +11701,11 @@
           <t>10–50 L/ha</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Use higher rates for heavy clay</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -11696,221 +11720,241 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
+          <t>foliar_vegetables</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
           <t>foliar</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>foliar</t>
-        </is>
-      </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>1 L per 100 L water</t>
+          <t>1 L per 100 L water, up to 5 L/ha</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Rate varies by crop</t>
+          <t>Weekly or as required</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>NSWL</t>
+          <t>636</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Nature's Soil Wetter - Liquid</t>
+          <t>Micronised Gypsum Liquid</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>lawn_garden</t>
+          <t>foliar_orchards_vineyards</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>spray</t>
+          <t>foliar</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>100 mL / 100 m²</t>
+          <t>1 L per 100 L water, up to 7 L/ha</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Do not shake</t>
+          <t>Every 2–4 weeks or as required</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>664</t>
+          <t>636</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Nature's Soil Wetter granules</t>
+          <t>Micronised Gypsum Liquid</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>lawns_gardens</t>
+          <t>foliar_ornamentals_turf</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>foliar</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>1.5–2 kg / 100 m² every 3–6 months</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr"/>
+          <t>1 L per 100 L water, up to 5 L/ha</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks or as required</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>664</t>
+          <t>636</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Nature's Soil Wetter granules</t>
+          <t>Micronised Gypsum Liquid</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>golf_greens</t>
+          <t>broadacre_crops_pasture</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>spray</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>1.5 kg / 100 m² every 1–2 months</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr"/>
+          <t>1–3 L/ha in 60–100 L water</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Depending on canopy closure</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>664</t>
+          <t>636</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Nature's Soil Wetter granules</t>
+          <t>Micronised Gypsum Liquid</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>fairways_sports</t>
+          <t>spot_spraying</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>spray</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>2 kg / 100 m² every 2–3 months</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr"/>
+          <t>50 mL per 10 L water</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Apply as required</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>664</t>
+          <t>636</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Nature's Soil Wetter granules</t>
+          <t>Micronised Gypsum Liquid</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>crops_vegetables</t>
+          <t>liquid_inject</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>inject</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>1.5–2 kg / 100 m²</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr"/>
+          <t>2–5 L/ha</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Minimum dilution 1:3</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>758</t>
+          <t>NSWL</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Neem Fertiliser Slow Release Granules</t>
+          <t>Nature's Soil Wetter - Liquid</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>soil_amendment</t>
+          <t>lawn_garden</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>spray</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>50–100 g/m²</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr"/>
+          <t>100 mL / 100 m²</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Do not shake</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>NSO</t>
+          <t>664</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Neem Seed Oil - 100% Cold Pressed virgin oil</t>
+          <t>Nature's Soil Wetter granules</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>garden</t>
+          <t>lawns_gardens</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>foliar</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>30 mL per 1 L water + a few drops biodegradable detergent</t>
+          <t>1.5–2 kg / 100 m² every 3–6 months</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr"/>
@@ -11918,59 +11962,55 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>NSO</t>
+          <t>664</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Neem Seed Oil - 100% Cold Pressed virgin oil</t>
+          <t>Nature's Soil Wetter granules</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>agriculture</t>
+          <t>golf_greens</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>spray</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>1 L neem oil per 200 L water</t>
-        </is>
-      </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>Apply 2–3 L prepared spray per hectare</t>
-        </is>
-      </c>
+          <t>1.5 kg / 100 m² every 1–2 months</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>29800</t>
+          <t>664</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Quantum H</t>
+          <t>Nature's Soil Wetter granules</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>home_garden</t>
+          <t>fairways_sports</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>spray</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>100 mL / 100 m²</t>
+          <t>2 kg / 100 m² every 2–3 months</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr"/>
@@ -11978,27 +12018,27 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>29782</t>
+          <t>664</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Rescue Remedy</t>
+          <t>Nature's Soil Wetter granules</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>crops_vegetables</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>spray</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>10 g / 10 L water or 10 g / 100 m²</t>
+          <t>1.5–2 kg / 100 m²</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr"/>
@@ -12006,17 +12046,17 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>1156</t>
+          <t>758</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Roots, Shoots &amp; Leaves - Granular</t>
+          <t>Neem Fertiliser Slow Release Granules</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>lawn</t>
+          <t>soil_amendment</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -12026,7 +12066,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>20–40 g/m²</t>
+          <t>50–100 g/m²</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr"/>
@@ -12034,27 +12074,27 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>1156</t>
+          <t>NSO</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Roots, Shoots &amp; Leaves - Granular</t>
+          <t>Neem Seed Oil - 100% Cold Pressed virgin oil</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>pots</t>
+          <t>garden</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>incorporate</t>
+          <t>foliar</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>4 g per litre of potting mix</t>
+          <t>30 mL per 1 L water + a few drops biodegradable detergent</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr"/>
@@ -12062,40 +12102,44 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>1156</t>
+          <t>NSO</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Roots, Shoots &amp; Leaves - Granular</t>
+          <t>Neem Seed Oil - 100% Cold Pressed virgin oil</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>plants_gardens</t>
+          <t>agriculture</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>spray</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>varies with plant type and size</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr"/>
+          <t>1 L neem oil per 200 L water</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Apply 2–3 L prepared spray per hectare</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>SWS</t>
+          <t>29800</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Seaweed Secrets</t>
+          <t>Quantum H</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -12118,17 +12162,17 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>STM</t>
+          <t>29782</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Stimulizer</t>
+          <t>Rescue Remedy</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>home_garden_area</t>
+          <t>general</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -12138,7 +12182,7 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>3 mL / 100 m²</t>
+          <t>10 g / 10 L water or 10 g / 100 m²</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr"/>
@@ -12146,27 +12190,27 @@
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>STM</t>
+          <t>1156</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Stimulizer</t>
+          <t>Roots, Shoots &amp; Leaves - Granular</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>watering_can</t>
+          <t>lawn</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>drench</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>2 mL per 9 L watering can</t>
+          <t>20–40 g/m²</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr"/>
@@ -12174,27 +12218,27 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>1156</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
+          <t>Roots, Shoots &amp; Leaves - Granular</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>lawn_garden</t>
+          <t>pots</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>incorporate</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>25–100 g/m²</t>
+          <t>4 g per litre of potting mix</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr"/>
@@ -12202,27 +12246,27 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>1156</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
+          <t>Roots, Shoots &amp; Leaves - Granular</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>potting_mix</t>
+          <t>plants_gardens</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>incorporate</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>5% by volume (~50 L per m³)</t>
+          <t>varies with plant type and size</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr"/>
@@ -12230,27 +12274,27 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>SWS</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
+          <t>Seaweed Secrets</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>soil_amendment</t>
+          <t>home_garden</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>spray</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>1–5 tonnes/ha</t>
+          <t>100 mL / 100 m²</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr"/>
@@ -12258,27 +12302,27 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>557</t>
+          <t>STM</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
+          <t>Stimulizer</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>tree_planting</t>
+          <t>home_garden_area</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>incorporate</t>
+          <t>spray</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>5–10 kg per planting hole or 3–5 kg per tree for trenching</t>
+          <t>3 mL / 100 m²</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr"/>
@@ -12286,27 +12330,27 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>WMP</t>
+          <t>STM</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Worm Magic Casting Pellets</t>
+          <t>Stimulizer</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>lawns_gardens</t>
+          <t>watering_can</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>drench</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>20–40 g/m²</t>
+          <t>2 mL per 9 L watering can</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr"/>
@@ -12314,91 +12358,83 @@
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>WMP</t>
+          <t>557</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Worm Magic Casting Pellets</t>
+          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>pots</t>
+          <t>lawn_garden</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>incorporate</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>2 tablespoons per 5 L potting mix</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>Every 4–6 weeks</t>
-        </is>
-      </c>
+          <t>25–100 g/m²</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>WMP</t>
+          <t>557</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Worm Magic Casting Pellets</t>
+          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>agriculture</t>
+          <t>potting_mix</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>incorporate</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>100–1000 kg/ha</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>Varies by crop</t>
-        </is>
-      </c>
+          <t>5% by volume (~50 L per m³)</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>WMB</t>
+          <t>557</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Worm Magic Liquid Compost Tea</t>
+          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>garden_beds_small_lawns</t>
+          <t>soil_amendment</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>drench</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>50–100 mL per 9 L water</t>
+          <t>1–5 tonnes/ha</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr"/>
@@ -12406,27 +12442,27 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>WMB</t>
+          <t>557</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Worm Magic Liquid Compost Tea</t>
+          <t>VolcaMin – Premium Clinoptilolite Zeolite</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>pots</t>
+          <t>tree_planting</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>drench</t>
+          <t>incorporate</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>10–20 mL per litre water</t>
+          <t>5–10 kg per planting hole or 3–5 kg per tree for trenching</t>
         </is>
       </c>
       <c r="F79" s="4" t="inlineStr"/>
@@ -12434,33 +12470,181 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>WMB</t>
+          <t>WMP</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Worm Magic Liquid Compost Tea</t>
+          <t>Worm Magic Casting Pellets</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>fruit_trees_shrubs</t>
+          <t>lawns_gardens</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>drench</t>
+          <t>spread</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>100–150 mL per 9 L water</t>
+          <t>20–40 g/m²</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>WMP</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Worm Magic Casting Pellets</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>pots</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>incorporate</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>2 tablespoons per 5 L potting mix</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Every 4–6 weeks</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>WMP</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Worm Magic Casting Pellets</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>agriculture</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>100–1000 kg/ha</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Varies by crop</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>WMB</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Worm Magic Liquid Compost Tea</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>garden_beds_small_lawns</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>drench</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>50–100 mL per 9 L water</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>WMB</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Worm Magic Liquid Compost Tea</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>pots</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>drench</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>10–20 mL per litre water</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>WMB</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Worm Magic Liquid Compost Tea</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>fruit_trees_shrubs</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>drench</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>100–150 mL per 9 L water</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F80"/>
+  <autoFilter ref="A1:F85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12474,7 +12658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX153"/>
+  <dimension ref="A1:AX162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34817,8 +35001,1200 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C154" s="4" t="inlineStr"/>
+      <c r="D154" s="4" t="inlineStr"/>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F154" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G154" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H154" s="4" t="inlineStr">
+        <is>
+          <t>Grass</t>
+        </is>
+      </c>
+      <c r="I154" s="4" t="inlineStr">
+        <is>
+          <t>Turf, lawns</t>
+        </is>
+      </c>
+      <c r="J154" s="4" t="inlineStr"/>
+      <c r="K154" s="4" t="inlineStr">
+        <is>
+          <t>500 mL / 100 m²</t>
+        </is>
+      </c>
+      <c r="L154" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks</t>
+        </is>
+      </c>
+      <c r="M154" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N154" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O154" s="4" t="inlineStr">
+        <is>
+          <t>Home garden: 45 mL in 9 L water; apply 1 L of mix per m² (500 mL product per 100 m²).</t>
+        </is>
+      </c>
+      <c r="P154" s="4" t="inlineStr"/>
+      <c r="Q154" s="4" t="inlineStr"/>
+      <c r="R154" s="4" t="inlineStr"/>
+      <c r="S154" s="4" t="inlineStr"/>
+      <c r="T154" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U154" s="4" t="inlineStr"/>
+      <c r="V154" s="4" t="inlineStr"/>
+      <c r="W154" s="4" t="inlineStr"/>
+      <c r="X154" s="4" t="inlineStr"/>
+      <c r="Y154" s="4" t="inlineStr"/>
+      <c r="Z154" s="4" t="inlineStr"/>
+      <c r="AA154" s="4" t="inlineStr"/>
+      <c r="AB154" s="4" t="inlineStr"/>
+      <c r="AC154" s="4" t="inlineStr"/>
+      <c r="AD154" s="4" t="inlineStr"/>
+      <c r="AE154" s="4" t="inlineStr"/>
+      <c r="AF154" s="4" t="inlineStr"/>
+      <c r="AG154" s="4" t="inlineStr"/>
+      <c r="AH154" s="4" t="inlineStr">
+        <is>
+          <t>500mL</t>
+        </is>
+      </c>
+      <c r="AI154" s="4" t="inlineStr">
+        <is>
+          <t>500mL</t>
+        </is>
+      </c>
+      <c r="AJ154" s="4" t="inlineStr"/>
+      <c r="AK154" s="4" t="inlineStr"/>
+      <c r="AL154" s="4" t="inlineStr"/>
+      <c r="AM154" s="4" t="inlineStr"/>
+      <c r="AN154" s="4" t="inlineStr">
+        <is>
+          <t>40mL</t>
+        </is>
+      </c>
+      <c r="AO154" s="4" t="inlineStr">
+        <is>
+          <t>40mL</t>
+        </is>
+      </c>
+      <c r="AP154" s="4" t="inlineStr">
+        <is>
+          <t>45mL</t>
+        </is>
+      </c>
+      <c r="AQ154" s="4" t="inlineStr">
+        <is>
+          <t>45mL</t>
+        </is>
+      </c>
+      <c r="AR154" s="4" t="inlineStr">
+        <is>
+          <t>50mL</t>
+        </is>
+      </c>
+      <c r="AS154" s="4" t="inlineStr">
+        <is>
+          <t>50mL</t>
+        </is>
+      </c>
+      <c r="AT154" s="4" t="inlineStr"/>
+      <c r="AU154" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV154" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW154" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks</t>
+        </is>
+      </c>
+      <c r="AX154" s="4" t="inlineStr">
+        <is>
+          <t>Home garden: 45 mL in 9 L water; apply 1 L of mix per m² (500 mL product per 100 m²).</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr"/>
+      <c r="D155" s="4" t="inlineStr"/>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F155" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G155" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H155" s="4" t="inlineStr">
+        <is>
+          <t>Home Garden</t>
+        </is>
+      </c>
+      <c r="I155" s="4" t="inlineStr">
+        <is>
+          <t>Gardens, lawns</t>
+        </is>
+      </c>
+      <c r="J155" s="4" t="inlineStr"/>
+      <c r="K155" s="4" t="inlineStr">
+        <is>
+          <t>500 mL / 100 m²</t>
+        </is>
+      </c>
+      <c r="L155" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks</t>
+        </is>
+      </c>
+      <c r="M155" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N155" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O155" s="4" t="inlineStr">
+        <is>
+          <t>45 mL in 9 L water; apply 1 L of mix per m².</t>
+        </is>
+      </c>
+      <c r="P155" s="4" t="inlineStr"/>
+      <c r="Q155" s="4" t="inlineStr"/>
+      <c r="R155" s="4" t="inlineStr"/>
+      <c r="S155" s="4" t="inlineStr"/>
+      <c r="T155" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U155" s="4" t="inlineStr"/>
+      <c r="V155" s="4" t="inlineStr"/>
+      <c r="W155" s="4" t="inlineStr"/>
+      <c r="X155" s="4" t="inlineStr"/>
+      <c r="Y155" s="4" t="inlineStr"/>
+      <c r="Z155" s="4" t="inlineStr"/>
+      <c r="AA155" s="4" t="inlineStr"/>
+      <c r="AB155" s="4" t="inlineStr"/>
+      <c r="AC155" s="4" t="inlineStr"/>
+      <c r="AD155" s="4" t="inlineStr"/>
+      <c r="AE155" s="4" t="inlineStr"/>
+      <c r="AF155" s="4" t="inlineStr"/>
+      <c r="AG155" s="4" t="inlineStr"/>
+      <c r="AH155" s="4" t="inlineStr">
+        <is>
+          <t>500mL</t>
+        </is>
+      </c>
+      <c r="AI155" s="4" t="inlineStr">
+        <is>
+          <t>500mL</t>
+        </is>
+      </c>
+      <c r="AJ155" s="4" t="inlineStr"/>
+      <c r="AK155" s="4" t="inlineStr"/>
+      <c r="AL155" s="4" t="inlineStr"/>
+      <c r="AM155" s="4" t="inlineStr"/>
+      <c r="AN155" s="4" t="inlineStr"/>
+      <c r="AO155" s="4" t="inlineStr"/>
+      <c r="AP155" s="4" t="inlineStr">
+        <is>
+          <t>45mL</t>
+        </is>
+      </c>
+      <c r="AQ155" s="4" t="inlineStr">
+        <is>
+          <t>45mL</t>
+        </is>
+      </c>
+      <c r="AR155" s="4" t="inlineStr"/>
+      <c r="AS155" s="4" t="inlineStr"/>
+      <c r="AT155" s="4" t="inlineStr"/>
+      <c r="AU155" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV155" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW155" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks</t>
+        </is>
+      </c>
+      <c r="AX155" s="4" t="inlineStr">
+        <is>
+          <t>45 mL in 9 L water; apply 1 L of mix per m².</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="inlineStr"/>
+      <c r="D156" s="4" t="inlineStr"/>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F156" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G156" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H156" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amelioration</t>
+        </is>
+      </c>
+      <c r="I156" s="4" t="inlineStr">
+        <is>
+          <t>Heavy clay</t>
+        </is>
+      </c>
+      <c r="J156" s="4" t="inlineStr"/>
+      <c r="K156" s="4" t="inlineStr"/>
+      <c r="L156" s="4" t="inlineStr">
+        <is>
+          <t>As required</t>
+        </is>
+      </c>
+      <c r="M156" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N156" s="4" t="inlineStr">
+        <is>
+          <t>Use higher rates for heavy clay (soil amelioration). Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O156" s="4" t="inlineStr">
+        <is>
+          <t>Soil ameliorant or fertigation 10–50 L/ha.</t>
+        </is>
+      </c>
+      <c r="P156" s="4" t="inlineStr"/>
+      <c r="Q156" s="4" t="inlineStr"/>
+      <c r="R156" s="4" t="inlineStr"/>
+      <c r="S156" s="4" t="inlineStr"/>
+      <c r="T156" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U156" s="4" t="inlineStr"/>
+      <c r="V156" s="4" t="inlineStr"/>
+      <c r="W156" s="4" t="inlineStr"/>
+      <c r="X156" s="4" t="inlineStr"/>
+      <c r="Y156" s="4" t="inlineStr"/>
+      <c r="Z156" s="4" t="inlineStr"/>
+      <c r="AA156" s="4" t="inlineStr"/>
+      <c r="AB156" s="4" t="inlineStr"/>
+      <c r="AC156" s="4" t="inlineStr"/>
+      <c r="AD156" s="4" t="inlineStr"/>
+      <c r="AE156" s="4" t="inlineStr"/>
+      <c r="AF156" s="4" t="inlineStr"/>
+      <c r="AG156" s="4" t="inlineStr"/>
+      <c r="AH156" s="4" t="inlineStr"/>
+      <c r="AI156" s="4" t="inlineStr"/>
+      <c r="AJ156" s="4" t="inlineStr"/>
+      <c r="AK156" s="4" t="inlineStr"/>
+      <c r="AL156" s="4" t="inlineStr">
+        <is>
+          <t>10L</t>
+        </is>
+      </c>
+      <c r="AM156" s="4" t="inlineStr">
+        <is>
+          <t>50L</t>
+        </is>
+      </c>
+      <c r="AN156" s="4" t="inlineStr"/>
+      <c r="AO156" s="4" t="inlineStr"/>
+      <c r="AP156" s="4" t="inlineStr"/>
+      <c r="AQ156" s="4" t="inlineStr"/>
+      <c r="AR156" s="4" t="inlineStr"/>
+      <c r="AS156" s="4" t="inlineStr"/>
+      <c r="AT156" s="4" t="inlineStr"/>
+      <c r="AU156" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV156" s="4" t="inlineStr">
+        <is>
+          <t>Use higher rates for heavy clay (soil amelioration). Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW156" s="4" t="inlineStr">
+        <is>
+          <t>As required</t>
+        </is>
+      </c>
+      <c r="AX156" s="4" t="inlineStr">
+        <is>
+          <t>Soil ameliorant or fertigation 10–50 L/ha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr"/>
+      <c r="D157" s="4" t="inlineStr"/>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F157" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G157" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H157" s="4" t="inlineStr">
+        <is>
+          <t>Vegetables</t>
+        </is>
+      </c>
+      <c r="I157" s="4" t="inlineStr">
+        <is>
+          <t>Foliar</t>
+        </is>
+      </c>
+      <c r="J157" s="4" t="inlineStr">
+        <is>
+          <t>1:100</t>
+        </is>
+      </c>
+      <c r="K157" s="4" t="inlineStr"/>
+      <c r="L157" s="4" t="inlineStr">
+        <is>
+          <t>Weekly or as required</t>
+        </is>
+      </c>
+      <c r="M157" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N157" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O157" s="4" t="inlineStr">
+        <is>
+          <t>Foliar vegetables: 1 L per 100 L water, up to 5 L/ha equivalent.</t>
+        </is>
+      </c>
+      <c r="P157" s="4" t="inlineStr"/>
+      <c r="Q157" s="4" t="inlineStr"/>
+      <c r="R157" s="4" t="inlineStr"/>
+      <c r="S157" s="4" t="inlineStr"/>
+      <c r="T157" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U157" s="4" t="inlineStr">
+        <is>
+          <t>1000mL</t>
+        </is>
+      </c>
+      <c r="V157" s="4" t="inlineStr">
+        <is>
+          <t>1000mL</t>
+        </is>
+      </c>
+      <c r="W157" s="4" t="inlineStr"/>
+      <c r="X157" s="4" t="inlineStr"/>
+      <c r="Y157" s="4" t="inlineStr"/>
+      <c r="Z157" s="4" t="inlineStr"/>
+      <c r="AA157" s="4" t="inlineStr"/>
+      <c r="AB157" s="4" t="inlineStr"/>
+      <c r="AC157" s="4" t="inlineStr"/>
+      <c r="AD157" s="4" t="inlineStr"/>
+      <c r="AE157" s="4" t="inlineStr"/>
+      <c r="AF157" s="4" t="inlineStr"/>
+      <c r="AG157" s="4" t="inlineStr"/>
+      <c r="AH157" s="4" t="inlineStr"/>
+      <c r="AI157" s="4" t="inlineStr"/>
+      <c r="AJ157" s="4" t="inlineStr"/>
+      <c r="AK157" s="4" t="inlineStr"/>
+      <c r="AL157" s="4" t="inlineStr">
+        <is>
+          <t>5L</t>
+        </is>
+      </c>
+      <c r="AM157" s="4" t="inlineStr">
+        <is>
+          <t>5L</t>
+        </is>
+      </c>
+      <c r="AN157" s="4" t="inlineStr"/>
+      <c r="AO157" s="4" t="inlineStr"/>
+      <c r="AP157" s="4" t="inlineStr"/>
+      <c r="AQ157" s="4" t="inlineStr"/>
+      <c r="AR157" s="4" t="inlineStr"/>
+      <c r="AS157" s="4" t="inlineStr"/>
+      <c r="AT157" s="4" t="inlineStr"/>
+      <c r="AU157" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV157" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW157" s="4" t="inlineStr">
+        <is>
+          <t>Weekly or as required</t>
+        </is>
+      </c>
+      <c r="AX157" s="4" t="inlineStr">
+        <is>
+          <t>1:100</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C158" s="4" t="inlineStr"/>
+      <c r="D158" s="4" t="inlineStr"/>
+      <c r="E158" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F158" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G158" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H158" s="4" t="inlineStr">
+        <is>
+          <t>Vineyard</t>
+        </is>
+      </c>
+      <c r="I158" s="4" t="inlineStr">
+        <is>
+          <t>Orchards and vineyards</t>
+        </is>
+      </c>
+      <c r="J158" s="4" t="inlineStr">
+        <is>
+          <t>1:100</t>
+        </is>
+      </c>
+      <c r="K158" s="4" t="inlineStr"/>
+      <c r="L158" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks or as required</t>
+        </is>
+      </c>
+      <c r="M158" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N158" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O158" s="4" t="inlineStr">
+        <is>
+          <t>Foliar orchards and vineyards: 1 L per 100 L water, up to 7 L/ha equivalent.</t>
+        </is>
+      </c>
+      <c r="P158" s="4" t="inlineStr"/>
+      <c r="Q158" s="4" t="inlineStr"/>
+      <c r="R158" s="4" t="inlineStr"/>
+      <c r="S158" s="4" t="inlineStr"/>
+      <c r="T158" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U158" s="4" t="inlineStr">
+        <is>
+          <t>1000mL</t>
+        </is>
+      </c>
+      <c r="V158" s="4" t="inlineStr">
+        <is>
+          <t>1000mL</t>
+        </is>
+      </c>
+      <c r="W158" s="4" t="inlineStr"/>
+      <c r="X158" s="4" t="inlineStr"/>
+      <c r="Y158" s="4" t="inlineStr"/>
+      <c r="Z158" s="4" t="inlineStr"/>
+      <c r="AA158" s="4" t="inlineStr"/>
+      <c r="AB158" s="4" t="inlineStr"/>
+      <c r="AC158" s="4" t="inlineStr"/>
+      <c r="AD158" s="4" t="inlineStr"/>
+      <c r="AE158" s="4" t="inlineStr"/>
+      <c r="AF158" s="4" t="inlineStr"/>
+      <c r="AG158" s="4" t="inlineStr"/>
+      <c r="AH158" s="4" t="inlineStr"/>
+      <c r="AI158" s="4" t="inlineStr"/>
+      <c r="AJ158" s="4" t="inlineStr"/>
+      <c r="AK158" s="4" t="inlineStr"/>
+      <c r="AL158" s="4" t="inlineStr">
+        <is>
+          <t>7L</t>
+        </is>
+      </c>
+      <c r="AM158" s="4" t="inlineStr">
+        <is>
+          <t>7L</t>
+        </is>
+      </c>
+      <c r="AN158" s="4" t="inlineStr"/>
+      <c r="AO158" s="4" t="inlineStr"/>
+      <c r="AP158" s="4" t="inlineStr"/>
+      <c r="AQ158" s="4" t="inlineStr"/>
+      <c r="AR158" s="4" t="inlineStr"/>
+      <c r="AS158" s="4" t="inlineStr"/>
+      <c r="AT158" s="4" t="inlineStr"/>
+      <c r="AU158" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV158" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW158" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks or as required</t>
+        </is>
+      </c>
+      <c r="AX158" s="4" t="inlineStr">
+        <is>
+          <t>1:100</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr"/>
+      <c r="D159" s="4" t="inlineStr"/>
+      <c r="E159" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F159" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G159" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H159" s="4" t="inlineStr">
+        <is>
+          <t>Grass</t>
+        </is>
+      </c>
+      <c r="I159" s="4" t="inlineStr">
+        <is>
+          <t>Foliar ornamentals and turf</t>
+        </is>
+      </c>
+      <c r="J159" s="4" t="inlineStr">
+        <is>
+          <t>1:100</t>
+        </is>
+      </c>
+      <c r="K159" s="4" t="inlineStr"/>
+      <c r="L159" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks or as required</t>
+        </is>
+      </c>
+      <c r="M159" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N159" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O159" s="4" t="inlineStr">
+        <is>
+          <t>Foliar ornamentals and turf: 1 L per 100 L water, up to 5 L/ha equivalent.</t>
+        </is>
+      </c>
+      <c r="P159" s="4" t="inlineStr"/>
+      <c r="Q159" s="4" t="inlineStr"/>
+      <c r="R159" s="4" t="inlineStr"/>
+      <c r="S159" s="4" t="inlineStr"/>
+      <c r="T159" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U159" s="4" t="inlineStr">
+        <is>
+          <t>1000mL</t>
+        </is>
+      </c>
+      <c r="V159" s="4" t="inlineStr">
+        <is>
+          <t>1000mL</t>
+        </is>
+      </c>
+      <c r="W159" s="4" t="inlineStr"/>
+      <c r="X159" s="4" t="inlineStr"/>
+      <c r="Y159" s="4" t="inlineStr"/>
+      <c r="Z159" s="4" t="inlineStr"/>
+      <c r="AA159" s="4" t="inlineStr"/>
+      <c r="AB159" s="4" t="inlineStr"/>
+      <c r="AC159" s="4" t="inlineStr"/>
+      <c r="AD159" s="4" t="inlineStr"/>
+      <c r="AE159" s="4" t="inlineStr"/>
+      <c r="AF159" s="4" t="inlineStr"/>
+      <c r="AG159" s="4" t="inlineStr"/>
+      <c r="AH159" s="4" t="inlineStr"/>
+      <c r="AI159" s="4" t="inlineStr"/>
+      <c r="AJ159" s="4" t="inlineStr"/>
+      <c r="AK159" s="4" t="inlineStr"/>
+      <c r="AL159" s="4" t="inlineStr">
+        <is>
+          <t>5L</t>
+        </is>
+      </c>
+      <c r="AM159" s="4" t="inlineStr">
+        <is>
+          <t>5L</t>
+        </is>
+      </c>
+      <c r="AN159" s="4" t="inlineStr"/>
+      <c r="AO159" s="4" t="inlineStr"/>
+      <c r="AP159" s="4" t="inlineStr"/>
+      <c r="AQ159" s="4" t="inlineStr"/>
+      <c r="AR159" s="4" t="inlineStr"/>
+      <c r="AS159" s="4" t="inlineStr"/>
+      <c r="AT159" s="4" t="inlineStr"/>
+      <c r="AU159" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV159" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW159" s="4" t="inlineStr">
+        <is>
+          <t>Every 2–4 weeks or as required</t>
+        </is>
+      </c>
+      <c r="AX159" s="4" t="inlineStr">
+        <is>
+          <t>1:100</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr"/>
+      <c r="D160" s="4" t="inlineStr"/>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H160" s="4" t="inlineStr">
+        <is>
+          <t>Broadacre Crops</t>
+        </is>
+      </c>
+      <c r="I160" s="4" t="inlineStr">
+        <is>
+          <t>Crops and pasture</t>
+        </is>
+      </c>
+      <c r="J160" s="4" t="inlineStr"/>
+      <c r="K160" s="4" t="inlineStr"/>
+      <c r="L160" s="4" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="M160" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N160" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O160" s="4" t="inlineStr">
+        <is>
+          <t>1–3 L/ha in 60–100 L water depending on canopy closure.</t>
+        </is>
+      </c>
+      <c r="P160" s="4" t="inlineStr"/>
+      <c r="Q160" s="4" t="inlineStr"/>
+      <c r="R160" s="4" t="inlineStr"/>
+      <c r="S160" s="4" t="inlineStr"/>
+      <c r="T160" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U160" s="4" t="inlineStr"/>
+      <c r="V160" s="4" t="inlineStr"/>
+      <c r="W160" s="4" t="inlineStr"/>
+      <c r="X160" s="4" t="inlineStr"/>
+      <c r="Y160" s="4" t="inlineStr"/>
+      <c r="Z160" s="4" t="inlineStr"/>
+      <c r="AA160" s="4" t="inlineStr"/>
+      <c r="AB160" s="4" t="inlineStr"/>
+      <c r="AC160" s="4" t="inlineStr"/>
+      <c r="AD160" s="4" t="inlineStr"/>
+      <c r="AE160" s="4" t="inlineStr"/>
+      <c r="AF160" s="4" t="inlineStr"/>
+      <c r="AG160" s="4" t="inlineStr"/>
+      <c r="AH160" s="4" t="inlineStr"/>
+      <c r="AI160" s="4" t="inlineStr"/>
+      <c r="AJ160" s="4" t="inlineStr"/>
+      <c r="AK160" s="4" t="inlineStr"/>
+      <c r="AL160" s="4" t="inlineStr">
+        <is>
+          <t>1L</t>
+        </is>
+      </c>
+      <c r="AM160" s="4" t="inlineStr">
+        <is>
+          <t>3L</t>
+        </is>
+      </c>
+      <c r="AN160" s="4" t="inlineStr"/>
+      <c r="AO160" s="4" t="inlineStr"/>
+      <c r="AP160" s="4" t="inlineStr"/>
+      <c r="AQ160" s="4" t="inlineStr"/>
+      <c r="AR160" s="4" t="inlineStr"/>
+      <c r="AS160" s="4" t="inlineStr"/>
+      <c r="AT160" s="4" t="inlineStr"/>
+      <c r="AU160" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV160" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW160" s="4" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="AX160" s="4" t="inlineStr">
+        <is>
+          <t>1–3 L/ha in 60–100 L water depending on canopy closure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr"/>
+      <c r="D161" s="4" t="inlineStr"/>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F161" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G161" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H161" s="4" t="inlineStr">
+        <is>
+          <t>Home Garden</t>
+        </is>
+      </c>
+      <c r="I161" s="4" t="inlineStr">
+        <is>
+          <t>Spot-spraying</t>
+        </is>
+      </c>
+      <c r="J161" s="4" t="inlineStr"/>
+      <c r="K161" s="4" t="inlineStr"/>
+      <c r="L161" s="4" t="inlineStr">
+        <is>
+          <t>As required</t>
+        </is>
+      </c>
+      <c r="M161" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N161" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O161" s="4" t="inlineStr">
+        <is>
+          <t>Spot-spraying: 50 mL per 10 L water.</t>
+        </is>
+      </c>
+      <c r="P161" s="4" t="inlineStr"/>
+      <c r="Q161" s="4" t="inlineStr"/>
+      <c r="R161" s="4" t="inlineStr"/>
+      <c r="S161" s="4" t="inlineStr"/>
+      <c r="T161" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U161" s="4" t="inlineStr"/>
+      <c r="V161" s="4" t="inlineStr"/>
+      <c r="W161" s="4" t="inlineStr"/>
+      <c r="X161" s="4" t="inlineStr"/>
+      <c r="Y161" s="4" t="inlineStr"/>
+      <c r="Z161" s="4" t="inlineStr"/>
+      <c r="AA161" s="4" t="inlineStr"/>
+      <c r="AB161" s="4" t="inlineStr"/>
+      <c r="AC161" s="4" t="inlineStr"/>
+      <c r="AD161" s="4" t="inlineStr"/>
+      <c r="AE161" s="4" t="inlineStr"/>
+      <c r="AF161" s="4" t="inlineStr"/>
+      <c r="AG161" s="4" t="inlineStr"/>
+      <c r="AH161" s="4" t="inlineStr"/>
+      <c r="AI161" s="4" t="inlineStr"/>
+      <c r="AJ161" s="4" t="inlineStr"/>
+      <c r="AK161" s="4" t="inlineStr"/>
+      <c r="AL161" s="4" t="inlineStr"/>
+      <c r="AM161" s="4" t="inlineStr"/>
+      <c r="AN161" s="4" t="inlineStr"/>
+      <c r="AO161" s="4" t="inlineStr"/>
+      <c r="AP161" s="4" t="inlineStr"/>
+      <c r="AQ161" s="4" t="inlineStr"/>
+      <c r="AR161" s="4" t="inlineStr">
+        <is>
+          <t>50mL</t>
+        </is>
+      </c>
+      <c r="AS161" s="4" t="inlineStr">
+        <is>
+          <t>50mL</t>
+        </is>
+      </c>
+      <c r="AT161" s="4" t="inlineStr"/>
+      <c r="AU161" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV161" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW161" s="4" t="inlineStr">
+        <is>
+          <t>As required</t>
+        </is>
+      </c>
+      <c r="AX161" s="4" t="inlineStr">
+        <is>
+          <t>Spot-spraying: 50 mL per 10 L water.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>Micronised Gypsum Liquid</t>
+        </is>
+      </c>
+      <c r="C162" s="4" t="inlineStr"/>
+      <c r="D162" s="4" t="inlineStr"/>
+      <c r="E162" s="4" t="inlineStr">
+        <is>
+          <t>Soil Amendmenet</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>Liquid</t>
+        </is>
+      </c>
+      <c r="G162" s="4" t="inlineStr">
+        <is>
+          <t>Clay soils, lawns, gardens, turf, orchards, vineyards, ornamentals, broadacre crops and pasture</t>
+        </is>
+      </c>
+      <c r="H162" s="4" t="inlineStr">
+        <is>
+          <t>Liquid Inject</t>
+        </is>
+      </c>
+      <c r="I162" s="4" t="inlineStr"/>
+      <c r="J162" s="4" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="K162" s="4" t="inlineStr"/>
+      <c r="L162" s="4" t="inlineStr">
+        <is>
+          <t>As required</t>
+        </is>
+      </c>
+      <c r="M162" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="N162" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="O162" s="4" t="inlineStr">
+        <is>
+          <t>Liquid inject 2–5 L/ha. Minimum dilution 1-part product to 3-parts water.</t>
+        </is>
+      </c>
+      <c r="P162" s="4" t="inlineStr"/>
+      <c r="Q162" s="4" t="inlineStr"/>
+      <c r="R162" s="4" t="inlineStr"/>
+      <c r="S162" s="4" t="inlineStr"/>
+      <c r="T162" s="4" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="U162" s="4" t="inlineStr"/>
+      <c r="V162" s="4" t="inlineStr"/>
+      <c r="W162" s="4" t="inlineStr"/>
+      <c r="X162" s="4" t="inlineStr"/>
+      <c r="Y162" s="4" t="inlineStr"/>
+      <c r="Z162" s="4" t="inlineStr"/>
+      <c r="AA162" s="4" t="inlineStr"/>
+      <c r="AB162" s="4" t="inlineStr"/>
+      <c r="AC162" s="4" t="inlineStr"/>
+      <c r="AD162" s="4" t="inlineStr"/>
+      <c r="AE162" s="4" t="inlineStr"/>
+      <c r="AF162" s="4" t="inlineStr"/>
+      <c r="AG162" s="4" t="inlineStr"/>
+      <c r="AH162" s="4" t="inlineStr"/>
+      <c r="AI162" s="4" t="inlineStr"/>
+      <c r="AJ162" s="4" t="inlineStr"/>
+      <c r="AK162" s="4" t="inlineStr"/>
+      <c r="AL162" s="4" t="inlineStr">
+        <is>
+          <t>2L</t>
+        </is>
+      </c>
+      <c r="AM162" s="4" t="inlineStr">
+        <is>
+          <t>5L</t>
+        </is>
+      </c>
+      <c r="AN162" s="4" t="inlineStr"/>
+      <c r="AO162" s="4" t="inlineStr"/>
+      <c r="AP162" s="4" t="inlineStr"/>
+      <c r="AQ162" s="4" t="inlineStr"/>
+      <c r="AR162" s="4" t="inlineStr"/>
+      <c r="AS162" s="4" t="inlineStr"/>
+      <c r="AT162" s="4" t="inlineStr"/>
+      <c r="AU162" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plantdoctor.com.au/Plant-Doctor-Micronised-Gypsum-Liquid-Organic-Certified</t>
+        </is>
+      </c>
+      <c r="AV162" s="4" t="inlineStr">
+        <is>
+          <t>Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+        </is>
+      </c>
+      <c r="AW162" s="4" t="inlineStr">
+        <is>
+          <t>As required</t>
+        </is>
+      </c>
+      <c r="AX162" s="4" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AX153"/>
+  <autoFilter ref="A1:AX162"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Trim On this day notes so they don’t restate how often a product is applied.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/pd_master_application_guide.xlsx
+++ b/data/pd_master_application_guide.xlsx
@@ -1127,7 +1127,7 @@
       </c>
       <c r="R2" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: test pH and magnesium first. Wait 6 weeks before iron.</t>
+          <t>Test pH and magnesium first. Wait 6 weeks before iron.</t>
         </is>
       </c>
       <c r="S2" s="4" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="AK2" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: test pH and magnesium first. Wait 6 weeks before iron. | Test soil pH and magnesium levels before application. Apply evenly across the area and water in to help granules break down. Avoid over-application, as excessive use can create nutrient imbalances.</t>
+          <t>Test pH and magnesium first. Wait 6 weeks before iron. | Test soil pH and magnesium levels before application. Apply evenly across the area and water in to help granules break down. Avoid over-application, as excessive use can create nutrient imbalances.</t>
         </is>
       </c>
       <c r="AL2" s="4" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="R3" s="4" t="inlineStr">
         <is>
-          <t>Hose-on tonic with iron. Apply independently from other liquids. Offset ~2 weeks if alternating with MaxGreen.</t>
+          <t>Apply independently from other liquids. Offset ~2 weeks if alternating with MaxGreen.</t>
         </is>
       </c>
       <c r="S3" s="4" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="AK3" s="4" t="inlineStr">
         <is>
-          <t>Hose-on tonic with iron. Apply independently from other liquids. Offset ~2 weeks if alternating with MaxGreen. | HOSE ON: connect the hose-on bottle and spray evenly. For refills, reuse the bottle with 4 L or 10 L concentrate packs. Can also be added to EZFLO. CONCENTRATE: shake well, apply during the coolest part of the day, lightly water in. Apply separately from most liquid fertilisers and pesticides. | Use 1 L concentrate + water to make ~2 L ready‑to‑use. A 4L refill to provide 8 treatments based on a 50/50 mix with water for each refill. | Ready‑to‑use coverage: 2 L bottle ≈ 200 m²
+          <t>Apply independently from other liquids. Offset ~2 weeks if alternating with MaxGreen. | HOSE ON: connect the hose-on bottle and spray evenly. For refills, reuse the bottle with 4 L or 10 L concentrate packs. Can also be added to EZFLO. CONCENTRATE: shake well, apply during the coolest part of the day, lightly water in. Apply separately from most liquid fertilisers and pesticides. | Use 1 L concentrate + water to make ~2 L ready‑to‑use. A 4L refill to provide 8 treatments based on a 50/50 mix with water for each refill. | Ready‑to‑use coverage: 2 L bottle ≈ 200 m²
 Concentrate refills provide up to ~8 applications in a 2 L bottle when diluted 1:1 with water.
 Compatible with EZFLO fertigation systems for larger or irregular areas.
 Pre‑mixed formula combines nutrients, wetting agents, organic stimulants and trace elements; excellent for overall plant and soil health beyond turf.</t>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="R4" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: when soil tests show low pH. Wait 6 weeks before iron.</t>
+          <t>Apply when soil tests show low pH. Wait 6 weeks before iron.</t>
         </is>
       </c>
       <c r="S4" s="4" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="AK4" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: when soil tests show low pH. Wait 6 weeks before iron. | Spread evenly over the soil surface and water in well. Where possible, incorporate into the topsoil. Always perform a soil test before application to determine the correct rate. Wait 6 weeks before applying iron.</t>
+          <t>Apply when soil tests show low pH. Wait 6 weeks before iron. | Spread evenly over the soil surface and water in well. Where possible, incorporate into the topsoil. Always perform a soil test before application to determine the correct rate. Wait 6 weeks before applying iron.</t>
         </is>
       </c>
       <c r="AL4" s="4" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: trees and grapevines every 6–8 weeks. Apply on a different day from seaweed, humic, wetter and Activ8. May stain paths.</t>
+          <t>Trees and grapevines every 6–8 weeks. May stain paths.</t>
         </is>
       </c>
       <c r="S5" s="4" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="AK5" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: trees and grapevines every 6–8 weeks. Apply on a different day from seaweed, humic, wetter and Activ8. May stain paths. | Apply as a foliar spray or soil drench during the coolest part of the day. Can be mixed with Stimulizer, but should be applied separately from most other fertilisers and liquid products. Always perform a jar test before mixing. | Corrects iron chlorosis (yellowing due to iron deficiency) and boosts green colour.
+          <t>Trees and grapevines every 6–8 weeks. May stain paths. | Apply as a foliar spray or soil drench during the coolest part of the day. Can be mixed with Stimulizer, but should be applied separately from most other fertilisers and liquid products. Always perform a jar test before mixing. | Corrects iron chlorosis (yellowing due to iron deficiency) and boosts green colour.
 Can be used as foliar spray or soil drench.
 Iron should be applied separately from other fertilisers to avoid reactions; compatible with some humic products but test before mixing.
 Iron application may stain paths/clothes; apply in calm conditions.</t>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="R6" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly on vegetables; every 6–8 weeks on trees and vines. Skip summer if fungal issues. Mixable with Stimulizer only.</t>
+          <t>Fortnightly on vegetables; every 6–8 weeks on trees and vines. Skip summer if fungal issues. Mixable with Stimulizer only.</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="AK6" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly on vegetables; every 6–8 weeks on trees and vines. Skip summer if fungal issues. Mixable with Stimulizer only. | HOSE ON: connect bottle and spray evenly; refill with 4 L or 10 L concentrate; EZFLO compatible. CONCENTRATE: shake well, apply in the coolest part of the day, lightly water in. Apply separately from most liquid fertilisers and pesticides. Stimulizer is compatible for tank mixing. | Corrects iron deficiency and supports green colour and growth in turf &amp; ornamentals. Avoid mixing with incompatible products; add iron last after other liquids diluted. | Use during active growth to support greener foliage and nutrient uptake; adjust frequency based on plant response. | Iron helps correct chlorosis; nitrogen supports vigorous growth.</t>
+          <t>Fortnightly on vegetables; every 6–8 weeks on trees and vines. Skip summer if fungal issues. Mixable with Stimulizer only. | HOSE ON: connect bottle and spray evenly; refill with 4 L or 10 L concentrate; EZFLO compatible. CONCENTRATE: shake well, apply in the coolest part of the day, lightly water in. Apply separately from most liquid fertilisers and pesticides. Stimulizer is compatible for tank mixing. | Corrects iron deficiency and supports green colour and growth in turf &amp; ornamentals. Avoid mixing with incompatible products; add iron last after other liquids diluted. | Use during active growth to support greener foliage and nutrient uptake; adjust frequency based on plant response. | Iron helps correct chlorosis; nitrogen supports vigorous growth.</t>
         </is>
       </c>
       <c r="AL6" s="4" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="R8" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: mix gently, do not shake. Do not tank-mix with iron.</t>
+          <t>Mix gently, do not shake. Do not tank-mix with iron.</t>
         </is>
       </c>
       <c r="S8" s="8" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="AK8" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: mix gently, do not shake. Do not tank-mix with iron. | Mix gently before use, do not shake. Water in lightly after application to activate the product. Compatible with most fertilisers, although a jar test is recommended before mixing with acidic or sulphate-based products. | Plant‑based wetting agent and soil conditioner that improves infiltration, water retention, and soil structure in dry or hydrophobic soils.
+          <t>Mix gently, do not shake. Do not tank-mix with iron. | Mix gently before use, do not shake. Water in lightly after application to activate the product. Compatible with most fertilisers, although a jar test is recommended before mixing with acidic or sulphate-based products. | Plant‑based wetting agent and soil conditioner that improves infiltration, water retention, and soil structure in dry or hydrophobic soils.
 Safe for all plants including natives and edibles; compatible with most fertilisers (jar test recommended first).
 Can be used as adjuvant with foliar/soil feeds to improve uptake and reduce water run‑off.</t>
         </is>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="R9" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly year-round. Can tank-mix with iron. Use at very low rates.</t>
+          <t>Can tank-mix with iron. Use at very low rates.</t>
         </is>
       </c>
       <c r="S9" s="8" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="AK9" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly year-round. Can tank-mix with iron. Use at very low rates. | Apply as a soil drench, foliar spray, hydroponic additive or mixed with fertilisers and other liquid inputs. Compatible with acidic and alkaline materials. Does not burn plants, lawns or soil if over-applied, but best results are at recommended rates. The only product the guide says can be safely mixed with iron. | Stimulizer enhances root development, nutrient uptake, soil microbial activity, stress resistance and overall plant vigor. It is compatible with other liquid fertilisers and tank mixes (perform a jar test first). Also used in hydroponics at lower per‑L rates</t>
+          <t>Can tank-mix with iron. Use at very low rates. | Apply as a soil drench, foliar spray, hydroponic additive or mixed with fertilisers and other liquid inputs. Compatible with acidic and alkaline materials. Does not burn plants, lawns or soil if over-applied, but best results are at recommended rates. The only product the guide says can be safely mixed with iron. | Stimulizer enhances root development, nutrient uptake, soil microbial activity, stress resistance and overall plant vigor. It is compatible with other liquid fertilisers and tank mixes (perform a jar test first). Also used in hydroponics at lower per‑L rates</t>
         </is>
       </c>
       <c r="AL9" s="4" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="R10" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly through the growing season; year-round for plant and soil health. Mixable with Stimulizer and most non-iron feeds.</t>
+          <t>Mixable with Stimulizer and most non-iron feeds.</t>
         </is>
       </c>
       <c r="S10" s="8" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="AK10" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly through the growing season; year-round for plant and soil health. Mixable with Stimulizer and most non-iron feeds. | Apply as a soil drench, foliar spray, fertigation or through sprinkler/drip irrigation. Can be mixed with most fertilisers and soil conditioners. When applying to foliage, check for staining on sensitive plants first. | Seaweed extract with added humic &amp; fulvic acids, rich in minerals and plant growth stimulants.
+          <t>Mixable with Stimulizer and most non-iron feeds. | Apply as a soil drench, foliar spray, fertigation or through sprinkler/drip irrigation. Can be mixed with most fertilisers and soil conditioners. When applying to foliage, check for staining on sensitive plants first. | Seaweed extract with added humic &amp; fulvic acids, rich in minerals and plant growth stimulants.
 Compatible with most fertilisers and soil conditioners; do not mix with iron products.
 Can be used across lawns, garden beds, vegetables, trees and broadacre crops. | For natives and other sensitive plants, use Seaweed Secrets and Activ8Mate at half strength.</t>
         </is>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="R11" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: more often during stress or transplanting. Do not tank-mix with iron (humic/fulvic).</t>
+          <t>More often during stress or transplanting. Do not tank-mix with iron (humic/fulvic).</t>
         </is>
       </c>
       <c r="S11" s="8" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="AK11" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: more often during stress or transplanting. Do not tank-mix with iron (humic/fulvic). | Apply as a soil drench, foliar spray, fertigation or irrigation. For best results on lawns, apply after mowing and water into the soil. Contains humic and fulvic acids — do not tank-mix with iron. | Lawn foliar/soil rate 9–12 L/ha (90–120 mL/100 m²). Apply evenly after mowing. Do not tank-mix with iron. | Garden beds and small lawns: 50–100 mL per 9 L water. Containers: 10–20 mL per 1 L water every 2–4 weeks. Fruit trees and shrubs: 100–150 mL per 9 L around the drip line every 4–6 weeks. | Horticulture foliar 5–7 L/ha. Fruit trees and shrubs at hobby rate 100–150 mL per 9 L around the drip line. | Pastures, broadacre, and fertigation 10–20 L/ha.</t>
+          <t>More often during stress or transplanting. Do not tank-mix with iron (humic/fulvic). | Apply as a soil drench, foliar spray, fertigation or irrigation. For best results on lawns, apply after mowing and water into the soil. Contains humic and fulvic acids — do not tank-mix with iron. | Lawn foliar/soil rate 9–12 L/ha (90–120 mL/100 m²). Apply evenly after mowing. Do not tank-mix with iron. | Garden beds and small lawns: 50–100 mL per 9 L water. Containers: 10–20 mL per 1 L water every 2–4 weeks. Fruit trees and shrubs: 100–150 mL per 9 L around the drip line every 4–6 weeks. | Horticulture foliar 5–7 L/ha. Fruit trees and shrubs at hobby rate 100–150 mL per 9 L around the drip line. | Pastures, broadacre, and fertigation 10–20 L/ha.</t>
         </is>
       </c>
       <c r="AL11" s="4" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="R12" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: pots every 4–6 weeks; lawns/beds as an ongoing soil-health dressing. Water in after spreading.</t>
+          <t>Pots every 4–6 weeks.</t>
         </is>
       </c>
       <c r="S12" s="4" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="AK12" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: pots every 4–6 weeks; lawns/beds as an ongoing soil-health dressing. Water in after spreading. | Apply evenly around plants, garden beds or lawn areas and water in after application to activate. Can be incorporated into soil, applied as a top dress or placed directly into planting holes for trees and vines. | Distribute evenly across lawn and garden areas and water in thoroughly. Typical home rate 20–40 g/m² (2–4 kg/100 m²). | Spread around plants, shrubs, or garden beds at 20–40 g/m². For pots: 2 tablespoons per 5 L potting mix, worked into the top layer. | Horticulture 250–1000 kg/ha. Apply along the drip line, into the planting hole, or as an even broadcast. | Broadacre and pastures 100–250 kg/ha. Band about 5 cm below the surface at sowing, or broadcast as a top-dress.</t>
+          <t>Pots every 4–6 weeks. | Apply evenly around plants, garden beds or lawn areas and water in after application to activate. Can be incorporated into soil, applied as a top dress or placed directly into planting holes for trees and vines. | Distribute evenly across lawn and garden areas and water in thoroughly. Typical home rate 20–40 g/m² (2–4 kg/100 m²). | Spread around plants, shrubs, or garden beds at 20–40 g/m². For pots: 2 tablespoons per 5 L potting mix, worked into the top layer. | Horticulture 250–1000 kg/ha. Apply along the drip line, into the planting hole, or as an even broadcast. | Broadacre and pastures 100–250 kg/ha. Band about 5 cm below the surface at sowing, or broadcast as a top-dress.</t>
         </is>
       </c>
       <c r="AL12" s="4" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: compacted, clay or sodic soils; soil prep or an ongoing soil program. Water in after spreading.</t>
+          <t>For compacted, clay or sodic soils.</t>
         </is>
       </c>
       <c r="S13" s="4" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="AK13" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: compacted, clay or sodic soils; soil prep or an ongoing soil program. Water in after spreading. | Apply evenly across the soil surface and water in after application to assist movement into the soil profile. Suitable for lawns, gardens, landscaping, parks, ovals and agricultural applications. | Provides slow-release calcium sulphate to improve soil structure, reduce compaction, and enhance nutrient availability.
+          <t>For compacted, clay or sodic soils. | Apply evenly across the soil surface and water in after application to assist movement into the soil profile. Suitable for lawns, gardens, landscaping, parks, ovals and agricultural applications. | Provides slow-release calcium sulphate to improve soil structure, reduce compaction, and enhance nutrient availability.
 Ideal for clay soils, compacted sites, lawns, garden beds, landscapes, and larger soil amelioration projects.
  Best used in conjunction with soil analysis and balanced nutrition plan.</t>
         </is>
@@ -3452,11 +3452,7 @@
           <t>spread</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr">
-        <is>
-          <t>Usage guide: every 3 months year-round. Water in after spreading.</t>
-        </is>
-      </c>
+      <c r="R14" s="4" t="inlineStr"/>
       <c r="S14" s="4" t="inlineStr">
         <is>
           <t>0</t>
@@ -3545,7 +3541,7 @@
       </c>
       <c r="AK14" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: every 3 months year-round. Water in after spreading. | Apply evenly around the plant root zone or across turf areas and water in after application. Suitable for lawns, vegetables, fruit trees, ornamentals, shrubs, natives and potted plants. Can be used with liquid fertilisers and soil conditioners. | Slow-release fertiliser feeding nitrogen, potassium and trace elements for sustained growth up to several months. Adjust based on turf vigour and soil conditions. | Works as a slow-release base in potting mixes. | Higher rates recommended for dense flowers/foliage. | Different rates for small/medium/large shrubs and trees; adjust to canopy size. | Balanced nutrition supports leafy and fruiting stages.</t>
+          <t>Apply evenly around the plant root zone or across turf areas and water in after application. Suitable for lawns, vegetables, fruit trees, ornamentals, shrubs, natives and potted plants. Can be used with liquid fertilisers and soil conditioners. | Slow-release fertiliser feeding nitrogen, potassium and trace elements for sustained growth up to several months. Adjust based on turf vigour and soil conditions. | Works as a slow-release base in potting mixes. | Higher rates recommended for dense flowers/foliage. | Different rates for small/medium/large shrubs and trees; adjust to canopy size. | Balanced nutrition supports leafy and fruiting stages.</t>
         </is>
       </c>
       <c r="AL14" s="4" t="inlineStr">
@@ -3653,7 +3649,7 @@
       </c>
       <c r="R15" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: apply independently; extra applications during drought, heat, frost or transplant stress.</t>
+          <t>Apply independently. Extra applications during drought, heat, frost or transplant stress.</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
@@ -3745,7 +3741,7 @@
       </c>
       <c r="AK15" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: apply independently; extra applications during drought, heat, frost or transplant stress. | Dissolve completely in water before application. Suitable for foliar spraying, soil drenching, irrigation and fertigation. May not be compatible with acidic fertilisers such as calcium nitrate, liquid phosphates and sulphate-based trace elements. | Premium Ascophyllum nodosum seaweed bio‑stimulant packed with natural hormones, trace elements, amino acids, and carbohydrates to improve root growth, stress resilience and plant vigour.
+          <t>Apply independently. Extra applications during drought, heat, frost or transplant stress. | Dissolve completely in water before application. Suitable for foliar spraying, soil drenching, irrigation and fertigation. May not be compatible with acidic fertilisers such as calcium nitrate, liquid phosphates and sulphate-based trace elements. | Premium Ascophyllum nodosum seaweed bio‑stimulant packed with natural hormones, trace elements, amino acids, and carbohydrates to improve root growth, stress resilience and plant vigour.
 Works via foliar spray or irrigation/fertigation and suitable for lawns, gardens, orchard crops and broadacre use.</t>
         </is>
       </c>
@@ -3854,7 +3850,7 @@
       </c>
       <c r="R16" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly for home gardens. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
       <c r="S16" s="8" t="inlineStr">
@@ -3947,7 +3943,7 @@
       </c>
       <c r="AK16" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly for home gardens. Do not tank-mix with iron. | Can be applied as a soil drench, foliar-compatible input, fertigation, sprinkler/drip irrigation or mixed with liquid nutrients. Compatible with most fertilisers, pesticides, fungicides and biological inputs. Avoid mixing directly with iron-based products. | Quantum H is a liquid humic and fulvic acid soil conditioner that improves soil structure, nutrient availability, water retention, and microbial activity.
+          <t>Do not tank-mix with iron. | Can be applied as a soil drench, foliar-compatible input, fertigation, sprinkler/drip irrigation or mixed with liquid nutrients. Compatible with most fertilisers, pesticides, fungicides and biological inputs. Avoid mixing directly with iron-based products. | Quantum H is a liquid humic and fulvic acid soil conditioner that improves soil structure, nutrient availability, water retention, and microbial activity.
 Not compatible with iron‑based products — apply separately.
 Suitable for irrigation systems (sprinkler/drip) with small applications integrated per irrigation.</t>
         </is>
@@ -4053,7 +4049,7 @@
       </c>
       <c r="R17" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: as required at seeding, transplant, flowering or stress. Jar test before mixing. Do not tank-mix with iron.</t>
+          <t>Use at seeding, transplant, flowering or stress. Jar test before mixing. Do not tank-mix with iron.</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
@@ -4128,7 +4124,7 @@
       </c>
       <c r="AK17" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: as required at seeding, transplant, flowering or stress. Jar test before mixing. Do not tank-mix with iron. | Fully soluble powder suitable for fertigation, foliar sprays, soil drenches and hydroponic systems. Can be combined with fertilisers to improve nutrient efficiency. Always conduct a jar test before mixing with new products, especially selective herbicides. Store sealed and dry.</t>
+          <t>Use at seeding, transplant, flowering or stress. Jar test before mixing. Do not tank-mix with iron. | Fully soluble powder suitable for fertigation, foliar sprays, soil drenches and hydroponic systems. Can be combined with fertilisers to improve nutrient efficiency. Always conduct a jar test before mixing with new products, especially selective herbicides. Store sealed and dry.</t>
         </is>
       </c>
       <c r="AL17" s="4" t="inlineStr">
@@ -4236,7 +4232,7 @@
       </c>
       <c r="R18" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: weekly or fortnightly through the growing season. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
       <c r="S18" s="8" t="inlineStr">
@@ -4327,7 +4323,7 @@
       </c>
       <c r="AK18" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: weekly or fortnightly through the growing season. Do not tank-mix with iron. | Can be applied through soil, foliar sprays, fertigation or hydroponic systems. Compatible with most fertilisers, soil conditioners and crop inputs; always conduct a jar test before tank mixing. | Fulvic acid chelates soil nutrients and improves uptake, root growth and plant stress resistance. Compatible with most fertilisers, soil conditioners, foliar sprays and hydroponic systems; always jar test before mixing. Can be used at any time of the year on all soil types which grow plants; turf, lawns, golf greens, all home garden plants, sandy and clay soils, pot plants, vegetables, and fruit trees.</t>
+          <t>Do not tank-mix with iron. | Can be applied through soil, foliar sprays, fertigation or hydroponic systems. Compatible with most fertilisers, soil conditioners and crop inputs; always conduct a jar test before tank mixing. | Fulvic acid chelates soil nutrients and improves uptake, root growth and plant stress resistance. Compatible with most fertilisers, soil conditioners, foliar sprays and hydroponic systems; always jar test before mixing. Can be used at any time of the year on all soil types which grow plants; turf, lawns, golf greens, all home garden plants, sandy and clay soils, pot plants, vegetables, and fruit trees.</t>
         </is>
       </c>
       <c r="AL18" s="4" t="inlineStr">
@@ -4630,7 +4626,7 @@
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
-          <t>Soluble humic. Jar test before mixing. Do not tank-mix with iron.</t>
+          <t>Jar test before mixing. Do not tank-mix with iron.</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
@@ -4723,7 +4719,7 @@
       </c>
       <c r="AK20" s="4" t="inlineStr">
         <is>
-          <t>Soluble humic. Jar test before mixing. Do not tank-mix with iron. | Pre-mix powder in water before application to ensure complete dissolution. Apply as a soil drench, foliar spray or through fertigation. Can be used alongside fertilisers and biological inputs, but perform a jar test before mixing. | Humic acid improves soil structure, nutrient uptake, microbial activity, and water retention.
+          <t>Jar test before mixing. Do not tank-mix with iron. | Pre-mix powder in water before application to ensure complete dissolution. Apply as a soil drench, foliar spray or through fertigation. Can be used alongside fertilisers and biological inputs, but perform a jar test before mixing. | Humic acid improves soil structure, nutrient uptake, microbial activity, and water retention.
 Compatible with most fertilisers and crop inputs; always perform a jar test if mixing.
 Effective for soil detoxification and enhancing fertiliser performance.</t>
         </is>
@@ -4829,7 +4825,7 @@
       </c>
       <c r="R21" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: at the start of growth or when leaves yellow. Preferred on alkaline soils. Apply independently.</t>
+          <t>Use at the start of growth or when leaves yellow. Preferred on alkaline soils.</t>
         </is>
       </c>
       <c r="S21" s="4" t="inlineStr">
@@ -4904,7 +4900,7 @@
       </c>
       <c r="AK21" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: at the start of growth or when leaves yellow. Preferred on alkaline soils. Apply independently. | Dissolve microgranules fully in water before application. Can be applied as a foliar spray, soil drench, pressure injection or through fertigation. Unlike iron sulphate, it is compatible with most fertilisers, but a jar test is recommended before mixing. Avoid contact with concrete and porous surfaces as staining may occur.</t>
+          <t>Use at the start of growth or when leaves yellow. Preferred on alkaline soils. | Dissolve microgranules fully in water before application. Can be applied as a foliar spray, soil drench, pressure injection or through fertigation. Unlike iron sulphate, it is compatible with most fertilisers, but a jar test is recommended before mixing. Avoid contact with concrete and porous surfaces as staining may occur.</t>
         </is>
       </c>
       <c r="AL21" s="4" t="inlineStr">
@@ -5012,7 +5008,7 @@
       </c>
       <c r="R22" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: planting, turf install or annual amendment. Does not break down.</t>
+          <t>Does not break down.</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
@@ -5101,7 +5097,7 @@
       </c>
       <c r="AK22" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: planting, turf install or annual amendment. Does not break down. | Incorporate into soil, potting mixes, compost blends or apply around root zones. Can be blended with fertilisers. &lt;1 mm powder: seed coatings, compost, fertigation, liquid suspension. 1–2 mm: potting mixes, gardens, seed raising. 2–4 mm: turf, landscaping, tree planting, drainage. | Natural zeolite improves soil structure, nutrient retention, water holding capacity, and reduces leaching.
+          <t>Does not break down. | Incorporate into soil, potting mixes, compost blends or apply around root zones. Can be blended with fertilisers. &lt;1 mm powder: seed coatings, compost, fertigation, liquid suspension. 1–2 mm: potting mixes, gardens, seed raising. 2–4 mm: turf, landscaping, tree planting, drainage. | Natural zeolite improves soil structure, nutrient retention, water holding capacity, and reduces leaching.
 Works in potting mixes, raised beds, gardens, turf, and broadacre soils.
 Can be mixed into fertiliser blends at 25–50 % of blend to enhance nutrient efficiency.</t>
         </is>
@@ -5505,7 +5501,7 @@
       </c>
       <c r="R25" s="4" t="inlineStr">
         <is>
-          <t>Garden flower/fruit granular. Not for lawns. Water in after spreading.</t>
+          <t>Garden flower/fruit granular. Not for lawns.</t>
         </is>
       </c>
       <c r="S25" s="4" t="inlineStr">
@@ -5596,7 +5592,7 @@
       </c>
       <c r="AK25" s="4" t="inlineStr">
         <is>
-          <t>Garden flower/fruit granular. Not for lawns. Water in after spreading. | Apply evenly around plants and water in well after application. Suitable for flowers, vegetables, herbs, fruit trees, ornamental plants and lawns. Use caution with phosphorus-sensitive natives such as grevilleas, banksias and proteas. | Application rates vary significantly with plant type; product is designed to support flowering, fruiting and root strength and is not intended for lawn nutrition (other products like MaxGreen or Lawn‑specific fertilisers are recommended for turf). Use caution with phosphorus‑sensitive natives — trial small areas first.</t>
+          <t>Garden flower/fruit granular. Not for lawns. | Apply evenly around plants and water in well after application. Suitable for flowers, vegetables, herbs, fruit trees, ornamental plants and lawns. Use caution with phosphorus-sensitive natives such as grevilleas, banksias and proteas. | Application rates vary significantly with plant type; product is designed to support flowering, fruiting and root strength and is not intended for lawn nutrition (other products like MaxGreen or Lawn‑specific fertilisers are recommended for turf). Use caution with phosphorus‑sensitive natives — trial small areas first.</t>
         </is>
       </c>
       <c r="AL25" s="4" t="inlineStr">
@@ -5700,7 +5696,7 @@
       </c>
       <c r="R26" s="4" t="inlineStr">
         <is>
-          <t>Home garden: 45 mL in 9 L water, apply 1 L/m² (500 mL per 100 m²) every 2–4 weeks. Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers.</t>
+          <t>Home garden: 45 mL in 9 L water, apply 1 L/m². Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers.</t>
         </is>
       </c>
       <c r="S26" s="4" t="inlineStr">
@@ -5795,7 +5791,7 @@
       </c>
       <c r="AK26" s="4" t="inlineStr">
         <is>
-          <t>Home garden: 45 mL in 9 L water, apply 1 L/m² (500 mL per 100 m²) every 2–4 weeks. Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers. | Shake or stir well before use and keep agitating. Pre-mix slowly. Will pass a 200-micron filter under ideal conditions; a coarse inline filter (500 micron / 35 mesh) is recommended. Drench with a watering can or equipment that can take larger particles. Not suitable for drippers. Foliar use can leave a visible residue on leaves and fruit. Jar test before mixing. Liquid inject minimum dilution 1-part product to 3-parts water. Store cool and keep sealed. | Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3. | Use higher rates for heavy clay (soil amelioration). Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
+          <t>Home garden: 45 mL in 9 L water, apply 1 L/m². Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers. | Shake or stir well before use and keep agitating. Pre-mix slowly. Will pass a 200-micron filter under ideal conditions; a coarse inline filter (500 micron / 35 mesh) is recommended. Drench with a watering can or equipment that can take larger particles. Not suitable for drippers. Foliar use can leave a visible residue on leaves and fruit. Jar test before mixing. Liquid inject minimum dilution 1-part product to 3-parts water. Store cool and keep sealed. | Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3. | Use higher rates for heavy clay (soil amelioration). Shake or stir well before use and keep agitating. Pre-mix slowly. Coarse inline filter (500 micron / 35 mesh) recommended. Drench with a watering can or equipment that can take larger particles; not for drippers. Foliar use can leave a visible residue. Jar test before mixing. Liquid inject minimum dilution 1:3.</t>
         </is>
       </c>
       <c r="AL26" s="4" t="inlineStr">
@@ -5903,7 +5899,7 @@
       </c>
       <c r="R27" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 3–6 months lawns; 2–3 months sports turf; 1–2 months greens. Reapply if water still beads.</t>
+          <t>3–6 months on lawns; 2–3 months on sports turf; 1–2 months on greens. Reapply if water still beads.</t>
         </is>
       </c>
       <c r="S27" s="4" t="inlineStr">
@@ -5992,7 +5988,7 @@
       </c>
       <c r="AK27" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 3–6 months lawns; 2–3 months sports turf; 1–2 months greens. Reapply if water still beads. | Apply evenly as a top-dress using a spreader or incorporate into potting mixes and garden beds. Watering after application is recommended to activate the granules, although not essential. Apply under tree drip lines or beneath mulch for fruit trees and natives. | Improves soil water infiltration, retention and uniform distribution in hydrophobic, compacted or nutrient‑poor soils.
+          <t>3–6 months on lawns; 2–3 months on sports turf; 1–2 months on greens. Reapply if water still beads. | Apply evenly as a top-dress using a spreader or incorporate into potting mixes and garden beds. Watering after application is recommended to activate the granules, although not essential. Apply under tree drip lines or beneath mulch for fruit trees and natives. | Improves soil water infiltration, retention and uniform distribution in hydrophobic, compacted or nutrient‑poor soils.
 Suitable for lawns, gardens, potting mixes, crops, pastures, fruit trees, natives and landscape soil conditioning.
 Can also be used for soil detoxification, microbe stimulation and sodium management.</t>
         </is>
@@ -6106,7 +6102,7 @@
       </c>
       <c r="R28" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly on vegetables; every 6–8 weeks on trees, fruit and vines.</t>
+          <t>Fortnightly on vegetables; every 6–8 weeks on trees, fruit and vines.</t>
         </is>
       </c>
       <c r="S28" s="8" t="inlineStr">
@@ -6197,7 +6193,7 @@
       </c>
       <c r="AK28" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly on vegetables; every 6–8 weeks on trees, fruit and vines. | Apply evenly to soil or foliage during the cooler parts of the day. Shake well before use. Suitable for flowers, vegetables, fruit trees, herbs, ornamental plants and turf. Use caution with phosphorus-sensitive native plants. | Excellent for flowering garden beds, ornamentals &amp; container plants. | Use throughout active vegetable growth for bloom and fruit set. | Supports flowering and fruit set on larger plants and orchard crops. | Designed for larger scale horticulture and broadacre use (e.g. orchards, vineyards).</t>
+          <t>Fortnightly on vegetables; every 6–8 weeks on trees, fruit and vines. | Apply evenly to soil or foliage during the cooler parts of the day. Shake well before use. Suitable for flowers, vegetables, fruit trees, herbs, ornamental plants and turf. Use caution with phosphorus-sensitive native plants. | Excellent for flowering garden beds, ornamentals &amp; container plants. | Use throughout active vegetable growth for bloom and fruit set. | Supports flowering and fruit set on larger plants and orchard crops. | Designed for larger scale horticulture and broadacre use (e.g. orchards, vineyards).</t>
         </is>
       </c>
       <c r="AL28" s="4" t="inlineStr">
@@ -6301,7 +6297,7 @@
       </c>
       <c r="R29" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 1–2 times per year; feeds up to 3 months. Ideal at renovation, before planting, or lawn recovery.</t>
+          <t>Feeds up to 3 months. Ideal at renovation, before planting, or lawn recovery.</t>
         </is>
       </c>
       <c r="S29" s="4" t="inlineStr">
@@ -6376,7 +6372,7 @@
       </c>
       <c r="AK29" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 1–2 times per year; feeds up to 3 months. Ideal at renovation, before planting, or lawn recovery. | Apply evenly over the soil surface and, where possible, incorporate into the top 10 cm of soil. Can be applied before sowing, laying turf, or swept into aeration holes. Water in lightly after application to activate the neem and soil wetter components.</t>
+          <t>Feeds up to 3 months. Ideal at renovation, before planting, or lawn recovery. | Apply evenly over the soil surface and, where possible, incorporate into the top 10 cm of soil. Can be applied before sowing, laying turf, or swept into aeration holes. Water in lightly after application to activate the neem and soil wetter components.</t>
         </is>
       </c>
       <c r="AL29" s="4" t="inlineStr">
@@ -6480,7 +6476,7 @@
       </c>
       <c r="R30" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: moss prevention every 6–8 weeks from late autumn through winter. Do not combine with lime.</t>
+          <t>For moss prevention</t>
         </is>
       </c>
       <c r="S30" s="4" t="inlineStr">
@@ -6555,7 +6551,7 @@
       </c>
       <c r="AK30" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: moss prevention every 6–8 weeks from late autumn through winter. Do not combine with lime. | Apply evenly using a broadcast spreader or dilute in water and spray. Water thoroughly after application. Avoid applying on windy days and wear protective gloves and a dust mask. Can stain concrete, paths and clothing.</t>
+          <t>For moss prevention | Apply evenly using a broadcast spreader or dilute in water and spray. Water thoroughly after application. Avoid applying on windy days and wear protective gloves and a dust mask. Can stain concrete, paths and clothing.</t>
         </is>
       </c>
       <c r="AL30" s="4" t="inlineStr">
@@ -6667,7 +6663,7 @@
       </c>
       <c r="R31" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: every 3 months year-round. Half rate in autumn and winter. Water in lightly.</t>
+          <t>Half rate in autumn and winter.</t>
         </is>
       </c>
       <c r="S31" s="4" t="inlineStr">
@@ -6756,7 +6752,7 @@
       </c>
       <c r="AK31" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: every 3 months year-round. Half rate in autumn and winter. Water in lightly. | Apply evenly using a broadcast spreader. Water in lightly after application to activate nutrients. Avoid applying during the heat of the day or when temperatures exceed 30°C. Suitable for residential lawns, fairways, tees, sports turf and professional turf applications. | Slow‑release feeding up to ~3 months; ideal after mowing or aeration.
+          <t>Half rate in autumn and winter. | Apply evenly using a broadcast spreader. Water in lightly after application to activate nutrients. Avoid applying during the heat of the day or when temperatures exceed 30°C. Suitable for residential lawns, fairways, tees, sports turf and professional turf applications. | Slow‑release feeding up to ~3 months; ideal after mowing or aeration.
 Water in lightly after application to activate nutrients.
 Can be used on lawns, turf, fairways, and around most plants (trial first if unsure).</t>
         </is>
@@ -6870,7 +6866,7 @@
       </c>
       <c r="R32" s="4" t="inlineStr">
         <is>
-          <t>Greens Grade for low-cut turf. Same 3-month interval as Fairway. Half rate in autumn and winter.</t>
+          <t>Greens Grade for low-cut turf. Half rate in autumn and winter.</t>
         </is>
       </c>
       <c r="S32" s="4" t="inlineStr">
@@ -6959,7 +6955,7 @@
       </c>
       <c r="AK32" s="4" t="inlineStr">
         <is>
-          <t>Greens Grade for low-cut turf. Same 3-month interval as Fairway. Half rate in autumn and winter. | Apply evenly using a suitable spreader for fine turf applications. The 1–2 mm mini-prill size provides excellent distribution across low-cut lawns, greens and high-performance turf. Lightly water after application to activate nutrients and minimise the risk of leaf burn. | Slow‑release formulation feeds turf consistently for up to ~3 months.
+          <t>Greens Grade for low-cut turf. Half rate in autumn and winter. | Apply evenly using a suitable spreader for fine turf applications. The 1–2 mm mini-prill size provides excellent distribution across low-cut lawns, greens and high-performance turf. Lightly water after application to activate nutrients and minimise the risk of leaf burn. | Slow‑release formulation feeds turf consistently for up to ~3 months.
 Ideal for maintaining dense, low‑cut turf and greens.
 Can also be used around beds and other lawn edges; conduct trial if unsure.</t>
         </is>
@@ -7073,7 +7069,7 @@
       </c>
       <c r="R33" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly when growing; once a month in cooler months. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
       <c r="S33" s="8" t="inlineStr">
@@ -7170,7 +7166,7 @@
       </c>
       <c r="AK33" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly when growing; once a month in cooler months. Do not tank-mix with iron. | Shake well before use. Apply evenly across lawns, gardens, vegetables, trees and natives. Light watering after application helps move nutrients into the soil and activate microbial processes. Suitable for foliar, soil and fertigation applications. Avoid mixing with iron products. | Use all year round; warmer months may benefit from more frequent, lighter applications.
+          <t>Do not tank-mix with iron. | Shake well before use. Apply evenly across lawns, gardens, vegetables, trees and natives. Light watering after application helps move nutrients into the soil and activate microbial processes. Suitable for foliar, soil and fertigation applications. Avoid mixing with iron products. | Use all year round; warmer months may benefit from more frequent, lighter applications.
 Apply half‑rate on natives, orchids, African violets, and ferns.
 Product enhances soil microbiology and plant nutrient uptake. | For natives and other sensitive plants, use Seaweed Secrets and Activ8Mate at half strength.</t>
         </is>
@@ -7284,7 +7280,7 @@
       </c>
       <c r="R34" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly in spring/summer; once a month in cooler months. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
       <c r="S34" s="8" t="inlineStr">
@@ -7379,7 +7375,7 @@
       </c>
       <c r="AK34" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly in spring/summer; once a month in cooler months. Do not tank-mix with iron. | Agitate well before use. Apply with sufficient water for even coverage and lightly water in if required. You can choose to lightly water in or leave on the leaf to dry prior to a light watering. Suitable for foliar, soil and fertigation applications. Compatible with most liquid fertilisers; always jar test before tank mixing. | Avoid mixing with iron products; trial patch first</t>
+          <t>Do not tank-mix with iron. | Agitate well before use. Apply with sufficient water for even coverage and lightly water in if required. You can choose to lightly water in or leave on the leaf to dry prior to a light watering. Suitable for foliar, soil and fertigation applications. Compatible with most liquid fertilisers; always jar test before tank mixing. | Avoid mixing with iron products; trial patch first</t>
         </is>
       </c>
       <c r="AL34" s="4" t="inlineStr">
@@ -7610,7 +7606,7 @@
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly in spring/summer; once a month in cooler months. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
     </row>
@@ -7697,7 +7693,7 @@
       </c>
       <c r="Q3" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly when growing; once a month in cooler months. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7780,7 @@
       </c>
       <c r="Q4" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: every 3 months year-round. Half rate in autumn and winter. Water in lightly.</t>
+          <t>Half rate in autumn and winter.</t>
         </is>
       </c>
     </row>
@@ -7871,7 +7867,7 @@
       </c>
       <c r="Q5" s="4" t="inlineStr">
         <is>
-          <t>Greens Grade for low-cut turf. Same 3-month interval as Fairway. Half rate in autumn and winter.</t>
+          <t>Greens Grade for low-cut turf. Half rate in autumn and winter.</t>
         </is>
       </c>
     </row>
@@ -7958,7 +7954,7 @@
       </c>
       <c r="Q6" s="4" t="inlineStr">
         <is>
-          <t>Garden flower/fruit granular. Not for lawns. Water in after spreading.</t>
+          <t>Garden flower/fruit granular. Not for lawns.</t>
         </is>
       </c>
     </row>
@@ -8045,7 +8041,7 @@
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly on vegetables; every 6–8 weeks on trees, fruit and vines.</t>
+          <t>Fortnightly on vegetables; every 6–8 weeks on trees, fruit and vines.</t>
         </is>
       </c>
     </row>
@@ -8132,7 +8128,7 @@
       </c>
       <c r="Q8" s="4" t="inlineStr">
         <is>
-          <t>Hose-on tonic with iron. Apply independently from other liquids. Offset ~2 weeks if alternating with MaxGreen.</t>
+          <t>Apply independently from other liquids. Offset ~2 weeks if alternating with MaxGreen.</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8215,7 @@
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: trees and grapevines every 6–8 weeks. Apply on a different day from seaweed, humic, wetter and Activ8. May stain paths.</t>
+          <t>Trees and grapevines every 6–8 weeks. May stain paths.</t>
         </is>
       </c>
     </row>
@@ -8306,7 +8302,7 @@
       </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly on vegetables; every 6–8 weeks on trees and vines. Skip summer if fungal issues. Mixable with Stimulizer only.</t>
+          <t>Fortnightly on vegetables; every 6–8 weeks on trees and vines. Skip summer if fungal issues. Mixable with Stimulizer only.</t>
         </is>
       </c>
     </row>
@@ -8393,7 +8389,7 @@
       </c>
       <c r="Q11" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 1–2 times per year; feeds up to 3 months. Ideal at renovation, before planting, or lawn recovery.</t>
+          <t>Feeds up to 3 months. Ideal at renovation, before planting, or lawn recovery.</t>
         </is>
       </c>
     </row>
@@ -8478,11 +8474,7 @@
           <t>Every 3 months</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
-        <is>
-          <t>Usage guide: every 3 months year-round. Water in after spreading.</t>
-        </is>
-      </c>
+      <c r="Q12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -8567,7 +8559,7 @@
       </c>
       <c r="Q13" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: weekly or fortnightly through the growing season. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
     </row>
@@ -8654,7 +8646,7 @@
       </c>
       <c r="Q14" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: compacted, clay or sodic soils; soil prep or an ongoing soil program. Water in after spreading.</t>
+          <t>For compacted, clay or sodic soils.</t>
         </is>
       </c>
     </row>
@@ -8828,7 +8820,7 @@
       </c>
       <c r="Q16" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: when soil tests show low pH. Wait 6 weeks before iron.</t>
+          <t>Apply when soil tests show low pH. Wait 6 weeks before iron.</t>
         </is>
       </c>
     </row>
@@ -8915,7 +8907,7 @@
       </c>
       <c r="Q17" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: 3–6 months lawns; 2–3 months sports turf; 1–2 months greens. Reapply if water still beads.</t>
+          <t>3–6 months on lawns; 2–3 months on sports turf; 1–2 months on greens. Reapply if water still beads.</t>
         </is>
       </c>
     </row>
@@ -9002,7 +8994,7 @@
       </c>
       <c r="Q18" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: mix gently, do not shake. Do not tank-mix with iron.</t>
+          <t>Mix gently, do not shake. Do not tank-mix with iron.</t>
         </is>
       </c>
     </row>
@@ -9089,7 +9081,7 @@
       </c>
       <c r="Q19" s="4" t="inlineStr">
         <is>
-          <t>Soluble humic. Jar test before mixing. Do not tank-mix with iron.</t>
+          <t>Jar test before mixing. Do not tank-mix with iron.</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9168,7 @@
       </c>
       <c r="Q20" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly for home gardens. Do not tank-mix with iron.</t>
+          <t>Do not tank-mix with iron.</t>
         </is>
       </c>
     </row>
@@ -9263,7 +9255,7 @@
       </c>
       <c r="Q21" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: apply independently; extra applications during drought, heat, frost or transplant stress.</t>
+          <t>Apply independently. Extra applications during drought, heat, frost or transplant stress.</t>
         </is>
       </c>
     </row>
@@ -9350,7 +9342,7 @@
       </c>
       <c r="Q22" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly through the growing season; year-round for plant and soil health. Mixable with Stimulizer and most non-iron feeds.</t>
+          <t>Mixable with Stimulizer and most non-iron feeds.</t>
         </is>
       </c>
     </row>
@@ -9437,7 +9429,7 @@
       </c>
       <c r="Q23" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: fortnightly year-round. Can tank-mix with iron. Use at very low rates.</t>
+          <t>Can tank-mix with iron. Use at very low rates.</t>
         </is>
       </c>
     </row>
@@ -9524,7 +9516,7 @@
       </c>
       <c r="Q24" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: planting, turf install or annual amendment. Does not break down.</t>
+          <t>Does not break down.</t>
         </is>
       </c>
     </row>
@@ -9611,7 +9603,7 @@
       </c>
       <c r="Q25" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: test pH and magnesium first. Wait 6 weeks before iron.</t>
+          <t>Test pH and magnesium first. Wait 6 weeks before iron.</t>
         </is>
       </c>
     </row>
@@ -9698,7 +9690,7 @@
       </c>
       <c r="Q26" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: moss prevention every 6–8 weeks from late autumn through winter. Do not combine with lime.</t>
+          <t>For moss prevention</t>
         </is>
       </c>
     </row>
@@ -9785,7 +9777,7 @@
       </c>
       <c r="Q27" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: at the start of growth or when leaves yellow. Preferred on alkaline soils. Apply independently.</t>
+          <t>Use at the start of growth or when leaves yellow. Preferred on alkaline soils.</t>
         </is>
       </c>
     </row>
@@ -9872,7 +9864,7 @@
       </c>
       <c r="Q28" s="4" t="inlineStr">
         <is>
-          <t>Home garden: 45 mL in 9 L water, apply 1 L/m² (500 mL per 100 m²) every 2–4 weeks. Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers.</t>
+          <t>Home garden: 45 mL in 9 L water, apply 1 L/m². Higher rates on heavy clay. Drench or use equipment that can take larger particles. Coarse 500-micron filter. Do not tank-mix with iron. Not for drippers.</t>
         </is>
       </c>
     </row>
@@ -9959,7 +9951,7 @@
       </c>
       <c r="Q29" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: as required at seeding, transplant, flowering or stress. Jar test before mixing. Do not tank-mix with iron.</t>
+          <t>Use at seeding, transplant, flowering or stress. Jar test before mixing. Do not tank-mix with iron.</t>
         </is>
       </c>
     </row>
@@ -10046,7 +10038,7 @@
       </c>
       <c r="Q30" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: pots every 4–6 weeks; lawns/beds as an ongoing soil-health dressing. Water in after spreading.</t>
+          <t>Pots every 4–6 weeks.</t>
         </is>
       </c>
     </row>
@@ -10133,7 +10125,7 @@
       </c>
       <c r="Q31" s="4" t="inlineStr">
         <is>
-          <t>Usage guide: more often during stress or transplanting. Do not tank-mix with iron (humic/fulvic).</t>
+          <t>More often during stress or transplanting. Do not tank-mix with iron (humic/fulvic).</t>
         </is>
       </c>
     </row>

</xml_diff>